<commit_message>
correcoes no projeto tendo em conta as alterações nos use cases
</commit_message>
<xml_diff>
--- a/assets/responsabilidades.xlsx
+++ b/assets/responsabilidades.xlsx
@@ -1600,7 +1600,7 @@
     <t xml:space="preserve">Atualizar lista encomendas</t>
   </si>
   <si>
-    <t xml:space="preserve">atualizarPecasEncomenda(id : int, pecas : List(Stock)) : void &amp;&amp; atualizarDataChegadaEncomenda(id : int, data_chegada : DateTime) : void &amp;&amp; atualizarDataPedidoEncomenda(id : int, data_pedido : DateTime) : void &amp;&amp; atualizarEstadoEncomenda(id : int, estado : EstadoEncomenda) : void</t>
+    <t xml:space="preserve">atualizarPecasEncomenda(id : int, pecas : List(Stock)) : void &amp;&amp; atualizarDataRececaoEncomenda(id : int, data_chegada : DateTime) : void &amp;&amp; atualizarDataEnvioEncomenda(id : int, data_pedido : DateTime) : void &amp;&amp; atualizarEstadoEncomenda(id : int, estado : EstadoEncomenda) : void</t>
   </si>
   <si>
     <t xml:space="preserve">(1) [Estado alterado de 'Rascunho' para 'Enviada'] (Passo 7)</t>
@@ -7361,7 +7361,7 @@
       <c r="D380" s="21"/>
       <c r="E380" s="11"/>
     </row>
-    <row r="381" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="381" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="2"/>
       <c r="B381" s="21" t="s">
         <v>486</v>
@@ -8432,7 +8432,7 @@
       <c r="D485" s="21"/>
       <c r="E485" s="11"/>
     </row>
-    <row r="486" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="486" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A486" s="2"/>
       <c r="B486" s="21"/>
       <c r="C486" s="21"/>

</xml_diff>

<commit_message>
update vpp e todo
</commit_message>
<xml_diff>
--- a/assets/responsabilidades.xlsx
+++ b/assets/responsabilidades.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="672">
   <si>
     <t xml:space="preserve">Use Case</t>
   </si>
@@ -714,6 +714,9 @@
     <t xml:space="preserve">removerReparacao(id: int) : bool</t>
   </si>
   <si>
+    <t xml:space="preserve">Este método deve meter a flag de disponibilidade da reparacao como false</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -905,6 +908,9 @@
   </si>
   <si>
     <t xml:space="preserve">removerPeca(id: int) : bool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quando o método é chamado deve meter a flag de disponibilidade da Peca a false</t>
   </si>
   <si>
     <r>
@@ -4569,7 +4575,7 @@
       <c r="D113" s="12"/>
       <c r="E113" s="12"/>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2"/>
       <c r="B114" s="10" t="s">
         <v>166</v>
@@ -4582,6 +4588,9 @@
       </c>
       <c r="E114" s="12" t="s">
         <v>138</v>
+      </c>
+      <c r="F114" s="18" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4594,7 +4603,7 @@
     <row r="116" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="6"/>
       <c r="B116" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C116" s="8"/>
       <c r="D116" s="9"/>
@@ -4612,7 +4621,7 @@
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="2"/>
       <c r="B118" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C118" s="11"/>
       <c r="D118" s="12"/>
@@ -4621,7 +4630,7 @@
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="2"/>
       <c r="B119" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C119" s="11"/>
       <c r="D119" s="12"/>
@@ -4630,22 +4639,22 @@
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="2"/>
       <c r="B120" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C120" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D120" s="12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E120" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2"/>
       <c r="B121" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C121" s="11"/>
       <c r="D121" s="12"/>
@@ -4654,7 +4663,7 @@
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2"/>
       <c r="B122" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C122" s="11"/>
       <c r="D122" s="12"/>
@@ -4663,67 +4672,67 @@
     <row r="123" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2"/>
       <c r="B123" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C123" s="11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D123" s="12" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E123" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2"/>
       <c r="B124" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C124" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D124" s="12" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E124" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2"/>
       <c r="B125" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C125" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D125" s="12" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E125" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="2"/>
       <c r="B126" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C126" s="11" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D126" s="12" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E126" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2"/>
       <c r="B127" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C127" s="11"/>
       <c r="D127" s="12"/>
@@ -4739,7 +4748,7 @@
     <row r="129" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="6"/>
       <c r="B129" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C129" s="8"/>
       <c r="D129" s="9"/>
@@ -4757,7 +4766,7 @@
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="2"/>
       <c r="B131" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C131" s="11"/>
       <c r="D131" s="12"/>
@@ -4766,22 +4775,22 @@
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2"/>
       <c r="B132" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C132" s="11" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D132" s="12" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E132" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2"/>
       <c r="B133" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C133" s="11"/>
       <c r="D133" s="12"/>
@@ -4790,7 +4799,7 @@
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="2"/>
       <c r="B134" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C134" s="11"/>
       <c r="D134" s="12"/>
@@ -4799,7 +4808,7 @@
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2"/>
       <c r="B135" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C135" s="11"/>
       <c r="D135" s="12"/>
@@ -4808,10 +4817,10 @@
     <row r="136" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2"/>
       <c r="B136" s="10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C136" s="11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D136" s="12"/>
       <c r="E136" s="12"/>
@@ -4819,10 +4828,10 @@
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2"/>
       <c r="B137" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C137" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D137" s="12"/>
       <c r="E137" s="12"/>
@@ -4830,10 +4839,10 @@
     <row r="138" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2"/>
       <c r="B138" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C138" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D138" s="12"/>
       <c r="E138" s="12"/>
@@ -4841,16 +4850,16 @@
     <row r="139" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2"/>
       <c r="B139" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C139" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D139" s="12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E139" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4863,7 +4872,7 @@
     <row r="141" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="6"/>
       <c r="B141" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C141" s="8"/>
       <c r="D141" s="9"/>
@@ -4881,22 +4890,22 @@
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="2"/>
       <c r="B143" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C143" s="11" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D143" s="12" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E143" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="2"/>
       <c r="B144" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C144" s="11"/>
       <c r="D144" s="12"/>
@@ -4905,7 +4914,7 @@
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="2"/>
       <c r="B145" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C145" s="11"/>
       <c r="D145" s="12"/>
@@ -4914,7 +4923,7 @@
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="2"/>
       <c r="B146" s="10" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C146" s="11"/>
       <c r="D146" s="12"/>
@@ -4923,16 +4932,19 @@
     <row r="147" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="2"/>
       <c r="B147" s="10" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C147" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D147" s="12" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E147" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
+      </c>
+      <c r="F147" s="18" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4946,7 +4958,7 @@
     <row r="149" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="6"/>
       <c r="B149" s="7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C149" s="8"/>
       <c r="D149" s="9"/>
@@ -4964,7 +4976,7 @@
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="2"/>
       <c r="B151" s="10" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C151" s="11"/>
       <c r="D151" s="12"/>
@@ -4973,7 +4985,7 @@
     <row r="152" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="2"/>
       <c r="B152" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C152" s="11"/>
       <c r="D152" s="12"/>
@@ -4982,22 +4994,22 @@
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="2"/>
       <c r="B153" s="10" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C153" s="11" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D153" s="12" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E153" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="2"/>
       <c r="B154" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C154" s="11"/>
       <c r="D154" s="12"/>
@@ -5006,7 +5018,7 @@
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="2"/>
       <c r="B155" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C155" s="11"/>
       <c r="D155" s="12"/>
@@ -5015,40 +5027,40 @@
     <row r="156" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="2"/>
       <c r="B156" s="10" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C156" s="11" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D156" s="12" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E156" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="2"/>
       <c r="B157" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C157" s="11" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D157" s="12" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E157" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="2"/>
       <c r="B158" s="10" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C158" s="11" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D158" s="12"/>
       <c r="E158" s="12"/>
@@ -5056,10 +5068,10 @@
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="2"/>
       <c r="B159" s="10" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C159" s="11" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D159" s="12"/>
       <c r="E159" s="12"/>
@@ -5067,16 +5079,16 @@
     <row r="160" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="2"/>
       <c r="B160" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C160" s="11" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D160" s="12" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E160" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5088,10 +5100,10 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B162" s="10" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C162" s="11"/>
       <c r="D162" s="12"/>
@@ -5100,7 +5112,7 @@
     <row r="163" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="2"/>
       <c r="B163" s="10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C163" s="11"/>
       <c r="D163" s="12"/>
@@ -5109,7 +5121,7 @@
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="2"/>
       <c r="B164" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C164" s="11"/>
       <c r="D164" s="12"/>
@@ -5118,37 +5130,37 @@
     <row r="165" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="2"/>
       <c r="B165" s="10" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C165" s="11" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D165" s="12" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E165" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="2"/>
       <c r="B166" s="10" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C166" s="11" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D166" s="12" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E166" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="2"/>
       <c r="B167" s="10" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C167" s="11"/>
       <c r="D167" s="12"/>
@@ -5164,7 +5176,7 @@
     <row r="169" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="6"/>
       <c r="B169" s="7" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C169" s="8"/>
       <c r="D169" s="9"/>
@@ -5182,7 +5194,7 @@
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="2"/>
       <c r="B171" s="10" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C171" s="11"/>
       <c r="D171" s="12"/>
@@ -5191,22 +5203,22 @@
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2"/>
       <c r="B172" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C172" s="11" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D172" s="12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E172" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2"/>
       <c r="B173" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C173" s="11"/>
       <c r="D173" s="12"/>
@@ -5215,7 +5227,7 @@
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2"/>
       <c r="B174" s="10" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C174" s="11"/>
       <c r="D174" s="12"/>
@@ -5224,7 +5236,7 @@
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="2"/>
       <c r="B175" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C175" s="11"/>
       <c r="D175" s="12"/>
@@ -5233,10 +5245,10 @@
     <row r="176" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="2"/>
       <c r="B176" s="10" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C176" s="11" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D176" s="12"/>
       <c r="E176" s="12"/>
@@ -5244,10 +5256,10 @@
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="2"/>
       <c r="B177" s="10" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C177" s="11" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D177" s="12"/>
       <c r="E177" s="12"/>
@@ -5255,10 +5267,10 @@
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="2"/>
       <c r="B178" s="10" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C178" s="11" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D178" s="12"/>
       <c r="E178" s="12"/>
@@ -5266,16 +5278,16 @@
     <row r="179" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="2"/>
       <c r="B179" s="10" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C179" s="11" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D179" s="12" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E179" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5288,7 +5300,7 @@
     <row r="181" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="6"/>
       <c r="B181" s="22" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C181" s="23"/>
       <c r="D181" s="23"/>
@@ -5306,7 +5318,7 @@
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="2"/>
       <c r="B183" s="21" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C183" s="21"/>
       <c r="D183" s="21"/>
@@ -5315,7 +5327,7 @@
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="2"/>
       <c r="B184" s="21" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C184" s="21"/>
       <c r="D184" s="21"/>
@@ -5324,10 +5336,10 @@
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="2"/>
       <c r="B185" s="21" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C185" s="21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D185" s="21"/>
       <c r="E185" s="11"/>
@@ -5335,7 +5347,7 @@
     <row r="186" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="2"/>
       <c r="B186" s="21" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C186" s="21"/>
       <c r="D186" s="21"/>
@@ -5344,7 +5356,7 @@
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="2"/>
       <c r="B187" s="21" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C187" s="21"/>
       <c r="D187" s="21"/>
@@ -5353,26 +5365,26 @@
     <row r="188" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="2"/>
       <c r="B188" s="21" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C188" s="21" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D188" s="21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E188" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F188" s="15"/>
     </row>
     <row r="189" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="2"/>
       <c r="B189" s="21" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C189" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D189" s="21"/>
       <c r="E189" s="11"/>
@@ -5380,55 +5392,55 @@
     <row r="190" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="2"/>
       <c r="B190" s="21" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C190" s="21" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D190" s="21" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E190" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="2"/>
       <c r="B191" s="21" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C191" s="21" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D191" s="21" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E191" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="2"/>
       <c r="B192" s="21" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C192" s="21" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D192" s="21" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E192" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F192" s="19" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="2"/>
       <c r="B193" s="21" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C193" s="21"/>
       <c r="D193" s="21"/>
@@ -5448,7 +5460,7 @@
     <row r="195" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="6"/>
       <c r="B195" s="22" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C195" s="23"/>
       <c r="D195" s="23"/>
@@ -5466,7 +5478,7 @@
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="2"/>
       <c r="B197" s="21" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C197" s="21"/>
       <c r="D197" s="21"/>
@@ -5475,7 +5487,7 @@
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="2"/>
       <c r="B198" s="21" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C198" s="21"/>
       <c r="D198" s="21"/>
@@ -5484,7 +5496,7 @@
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="2"/>
       <c r="B199" s="21" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C199" s="21"/>
       <c r="D199" s="21"/>
@@ -5493,7 +5505,7 @@
     <row r="200" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="2"/>
       <c r="B200" s="21" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C200" s="21"/>
       <c r="D200" s="21"/>
@@ -5502,7 +5514,7 @@
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="2"/>
       <c r="B201" s="21" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C201" s="21"/>
       <c r="D201" s="21"/>
@@ -5511,10 +5523,10 @@
     <row r="202" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="2"/>
       <c r="B202" s="21" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C202" s="21" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D202" s="21"/>
       <c r="E202" s="11"/>
@@ -5522,10 +5534,10 @@
     <row r="203" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="2"/>
       <c r="B203" s="21" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C203" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D203" s="21"/>
       <c r="E203" s="11"/>
@@ -5533,10 +5545,10 @@
     <row r="204" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="2"/>
       <c r="B204" s="21" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C204" s="21" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D204" s="21"/>
       <c r="E204" s="11"/>
@@ -5544,10 +5556,10 @@
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="2"/>
       <c r="B205" s="21" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C205" s="21" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D205" s="21"/>
       <c r="E205" s="11"/>
@@ -5555,7 +5567,7 @@
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="2"/>
       <c r="B206" s="21" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C206" s="21"/>
       <c r="D206" s="21"/>
@@ -5570,10 +5582,10 @@
     </row>
     <row r="208" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B208" s="21" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C208" s="21"/>
       <c r="D208" s="21"/>
@@ -5582,7 +5594,7 @@
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="2"/>
       <c r="B209" s="21" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C209" s="21"/>
       <c r="D209" s="21"/>
@@ -5591,25 +5603,25 @@
     <row r="210" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="2"/>
       <c r="B210" s="21" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C210" s="21" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D210" s="21" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E210" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F210" s="19" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="2"/>
       <c r="B211" s="21" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C211" s="21"/>
       <c r="D211" s="21"/>
@@ -5618,7 +5630,7 @@
     <row r="212" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="2"/>
       <c r="B212" s="21" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C212" s="21"/>
       <c r="D212" s="21"/>
@@ -5627,25 +5639,25 @@
     <row r="213" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="2"/>
       <c r="B213" s="21" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C213" s="21" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D213" s="21" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E213" s="11" t="s">
         <v>131</v>
       </c>
       <c r="F213" s="19" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="2"/>
       <c r="B214" s="21" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C214" s="21"/>
       <c r="D214" s="21"/>
@@ -5661,7 +5673,7 @@
     <row r="216" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="6"/>
       <c r="B216" s="22" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C216" s="23"/>
       <c r="D216" s="23"/>
@@ -5679,7 +5691,7 @@
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="2"/>
       <c r="B218" s="21" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C218" s="21"/>
       <c r="D218" s="21"/>
@@ -5688,22 +5700,22 @@
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="2"/>
       <c r="B219" s="21" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C219" s="21" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D219" s="21" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E219" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="2"/>
       <c r="B220" s="21" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C220" s="21"/>
       <c r="D220" s="21"/>
@@ -5712,22 +5724,22 @@
     <row r="221" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="2"/>
       <c r="B221" s="21" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C221" s="21" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D221" s="24" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E221" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="2"/>
       <c r="B222" s="21" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C222" s="21"/>
       <c r="D222" s="21"/>
@@ -5736,28 +5748,28 @@
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="2"/>
       <c r="B223" s="21" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C223" s="21" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D223" s="21" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E223" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="2"/>
       <c r="B224" s="21" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C224" s="21" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D224" s="21" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E224" s="11" t="s">
         <v>131</v>
@@ -5766,7 +5778,7 @@
     <row r="225" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="2"/>
       <c r="B225" s="21" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C225" s="21"/>
       <c r="D225" s="21"/>
@@ -5785,7 +5797,7 @@
     <row r="227" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="6"/>
       <c r="B227" s="22" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C227" s="23"/>
       <c r="D227" s="23"/>
@@ -5803,7 +5815,7 @@
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="2"/>
       <c r="B229" s="21" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C229" s="21"/>
       <c r="D229" s="21"/>
@@ -5812,7 +5824,7 @@
     <row r="230" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="2"/>
       <c r="B230" s="21" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C230" s="21"/>
       <c r="D230" s="21"/>
@@ -5821,7 +5833,7 @@
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="2"/>
       <c r="B231" s="21" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C231" s="21"/>
       <c r="D231" s="21"/>
@@ -5841,10 +5853,10 @@
     <row r="233" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="2"/>
       <c r="B233" s="21" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C233" s="21" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D233" s="21"/>
       <c r="E233" s="11"/>
@@ -5852,16 +5864,16 @@
     <row r="234" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="2"/>
       <c r="B234" s="21" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C234" s="21" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D234" s="21" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E234" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5874,7 +5886,7 @@
     <row r="236" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="6"/>
       <c r="B236" s="22" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C236" s="23"/>
       <c r="D236" s="23"/>
@@ -5892,7 +5904,7 @@
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="2"/>
       <c r="B238" s="21" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C238" s="21"/>
       <c r="D238" s="21"/>
@@ -5901,22 +5913,22 @@
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="2"/>
       <c r="B239" s="21" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C239" s="21" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D239" s="21" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E239" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="2"/>
       <c r="B240" s="21" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C240" s="21"/>
       <c r="D240" s="21"/>
@@ -5925,7 +5937,7 @@
     <row r="241" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="2"/>
       <c r="B241" s="21" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C241" s="21"/>
       <c r="D241" s="21"/>
@@ -5934,7 +5946,7 @@
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="2"/>
       <c r="B242" s="21" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C242" s="21"/>
       <c r="D242" s="21"/>
@@ -5943,7 +5955,7 @@
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="2"/>
       <c r="B243" s="21" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C243" s="21" t="s">
         <v>22</v>
@@ -5954,10 +5966,10 @@
     <row r="244" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="2"/>
       <c r="B244" s="21" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C244" s="21" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D244" s="21"/>
       <c r="E244" s="11"/>
@@ -5965,16 +5977,16 @@
     <row r="245" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="2"/>
       <c r="B245" s="21" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C245" s="21" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D245" s="21" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E245" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5987,7 +5999,7 @@
     <row r="247" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="6"/>
       <c r="B247" s="22" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C247" s="23"/>
       <c r="D247" s="23"/>
@@ -6005,7 +6017,7 @@
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="2"/>
       <c r="B249" s="21" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C249" s="21"/>
       <c r="D249" s="21"/>
@@ -6014,22 +6026,22 @@
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="2"/>
       <c r="B250" s="21" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C250" s="21" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D250" s="21" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E250" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="2"/>
       <c r="B251" s="21" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C251" s="21"/>
       <c r="D251" s="21"/>
@@ -6038,7 +6050,7 @@
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="2"/>
       <c r="B252" s="21" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C252" s="21"/>
       <c r="D252" s="21"/>
@@ -6047,16 +6059,16 @@
     <row r="253" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="2"/>
       <c r="B253" s="21" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C253" s="21" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D253" s="21" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E253" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6070,7 +6082,7 @@
     <row r="255" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="6"/>
       <c r="B255" s="22" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C255" s="23"/>
       <c r="D255" s="23"/>
@@ -6088,7 +6100,7 @@
     <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="2"/>
       <c r="B257" s="21" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C257" s="21"/>
       <c r="D257" s="21"/>
@@ -6097,7 +6109,7 @@
     <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="2"/>
       <c r="B258" s="21" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C258" s="21"/>
       <c r="D258" s="21"/>
@@ -6106,37 +6118,37 @@
     <row r="259" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="2"/>
       <c r="B259" s="21" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C259" s="21" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D259" s="24" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E259" s="25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="2"/>
       <c r="B260" s="21" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C260" s="21" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D260" s="21" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E260" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="261" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="2"/>
       <c r="B261" s="21" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C261" s="21"/>
       <c r="D261" s="21"/>
@@ -6145,7 +6157,7 @@
     <row r="262" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="2"/>
       <c r="B262" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C262" s="21"/>
       <c r="D262" s="21"/>
@@ -6154,7 +6166,7 @@
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="2"/>
       <c r="B263" s="21" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C263" s="21"/>
       <c r="D263" s="21"/>
@@ -6163,7 +6175,7 @@
     <row r="264" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="2"/>
       <c r="B264" s="21" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C264" s="21"/>
       <c r="D264" s="21"/>
@@ -6172,7 +6184,7 @@
     <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="2"/>
       <c r="B265" s="21" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C265" s="21"/>
       <c r="D265" s="21"/>
@@ -6181,10 +6193,10 @@
     <row r="266" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="2"/>
       <c r="B266" s="21" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C266" s="21" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D266" s="21"/>
       <c r="E266" s="11"/>
@@ -6192,16 +6204,16 @@
     <row r="267" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="2"/>
       <c r="B267" s="21" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="C267" s="21" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="D267" s="21" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="E267" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6214,7 +6226,7 @@
     <row r="269" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="6"/>
       <c r="B269" s="22" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C269" s="23"/>
       <c r="D269" s="23"/>
@@ -6232,7 +6244,7 @@
     <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="2"/>
       <c r="B271" s="21" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C271" s="21"/>
       <c r="D271" s="21"/>
@@ -6241,22 +6253,22 @@
     <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="2"/>
       <c r="B272" s="21" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C272" s="21" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="D272" s="21" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="E272" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="2"/>
       <c r="B273" s="21" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C273" s="21"/>
       <c r="D273" s="21"/>
@@ -6265,22 +6277,22 @@
     <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="2"/>
       <c r="B274" s="21" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C274" s="21" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D274" s="21" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E274" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="2"/>
       <c r="B275" s="21" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="C275" s="21"/>
       <c r="D275" s="21"/>
@@ -6289,7 +6301,7 @@
     <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="2"/>
       <c r="B276" s="21" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C276" s="21"/>
       <c r="D276" s="21"/>
@@ -6298,10 +6310,10 @@
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="2"/>
       <c r="B277" s="21" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C277" s="21" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D277" s="21"/>
       <c r="E277" s="11"/>
@@ -6309,16 +6321,16 @@
     <row r="278" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="2"/>
       <c r="B278" s="21" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C278" s="21" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D278" s="21" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="E278" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6330,10 +6342,10 @@
     </row>
     <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B280" s="21" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="C280" s="21"/>
       <c r="D280" s="21"/>
@@ -6342,7 +6354,7 @@
     <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="2"/>
       <c r="B281" s="21" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C281" s="21"/>
       <c r="D281" s="21"/>
@@ -6351,7 +6363,7 @@
     <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="2"/>
       <c r="B282" s="21" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C282" s="21"/>
       <c r="D282" s="21"/>
@@ -6360,10 +6372,10 @@
     <row r="283" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="2"/>
       <c r="B283" s="21" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="C283" s="21" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D283" s="21"/>
       <c r="E283" s="11"/>
@@ -6371,22 +6383,22 @@
     <row r="284" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="2"/>
       <c r="B284" s="21" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C284" s="21" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D284" s="21" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="E284" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="2"/>
       <c r="B285" s="21" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="C285" s="21"/>
       <c r="D285" s="21"/>
@@ -6395,7 +6407,7 @@
     <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="2"/>
       <c r="B286" s="21" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C286" s="21"/>
       <c r="D286" s="21"/>
@@ -6404,7 +6416,7 @@
     <row r="287" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="2"/>
       <c r="B287" s="21" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C287" s="21"/>
       <c r="D287" s="21"/>
@@ -6413,7 +6425,7 @@
     <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="2"/>
       <c r="B288" s="21" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C288" s="21"/>
       <c r="D288" s="21"/>
@@ -6422,10 +6434,10 @@
     <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="2"/>
       <c r="B289" s="21" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C289" s="21" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="D289" s="21"/>
       <c r="E289" s="11"/>
@@ -6433,10 +6445,10 @@
     <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="2"/>
       <c r="B290" s="21" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="C290" s="21" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="D290" s="21"/>
       <c r="E290" s="11"/>
@@ -6444,22 +6456,22 @@
     <row r="291" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="2"/>
       <c r="B291" s="21" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C291" s="21" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D291" s="21" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="E291" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="2"/>
       <c r="B292" s="21" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C292" s="21"/>
       <c r="D292" s="21"/>
@@ -6475,7 +6487,7 @@
     <row r="294" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A294" s="6"/>
       <c r="B294" s="22" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C294" s="23"/>
       <c r="D294" s="23"/>
@@ -6493,7 +6505,7 @@
     <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="2"/>
       <c r="B296" s="21" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C296" s="21"/>
       <c r="D296" s="21"/>
@@ -6502,7 +6514,7 @@
     <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A297" s="2"/>
       <c r="B297" s="21" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C297" s="21"/>
       <c r="D297" s="21"/>
@@ -6511,7 +6523,7 @@
     <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="2"/>
       <c r="B298" s="21" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="C298" s="21"/>
       <c r="D298" s="21"/>
@@ -6520,7 +6532,7 @@
     <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="2"/>
       <c r="B299" s="21" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C299" s="21"/>
       <c r="D299" s="21"/>
@@ -6529,16 +6541,16 @@
     <row r="300" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A300" s="2"/>
       <c r="B300" s="21" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="C300" s="21" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D300" s="21" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="E300" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6551,7 +6563,7 @@
     <row r="302" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A302" s="6"/>
       <c r="B302" s="22" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="C302" s="23"/>
       <c r="D302" s="23"/>
@@ -6569,7 +6581,7 @@
     <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A304" s="2"/>
       <c r="B304" s="21" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C304" s="21"/>
       <c r="D304" s="21"/>
@@ -6578,7 +6590,7 @@
     <row r="305" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="2"/>
       <c r="B305" s="21" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C305" s="21"/>
       <c r="D305" s="21"/>
@@ -6587,7 +6599,7 @@
     <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A306" s="2"/>
       <c r="B306" s="21" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C306" s="21"/>
       <c r="D306" s="21"/>
@@ -6607,7 +6619,7 @@
     <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A308" s="2"/>
       <c r="B308" s="21" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C308" s="21" t="s">
         <v>42</v>
@@ -6618,10 +6630,10 @@
     <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A309" s="2"/>
       <c r="B309" s="21" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C309" s="21" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D309" s="21"/>
       <c r="E309" s="11"/>
@@ -6629,7 +6641,7 @@
     <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A310" s="2"/>
       <c r="B310" s="21" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="C310" s="21" t="s">
         <v>51</v>
@@ -6640,16 +6652,16 @@
     <row r="311" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A311" s="2"/>
       <c r="B311" s="21" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="C311" s="21" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="D311" s="21" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="E311" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6662,7 +6674,7 @@
     <row r="313" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="6"/>
       <c r="B313" s="22" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C313" s="23"/>
       <c r="D313" s="23"/>
@@ -6680,7 +6692,7 @@
     <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A315" s="2"/>
       <c r="B315" s="21" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C315" s="21"/>
       <c r="D315" s="21"/>
@@ -6689,22 +6701,22 @@
     <row r="316" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A316" s="2"/>
       <c r="B316" s="21" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="C316" s="21" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D316" s="21" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="E316" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A317" s="2"/>
       <c r="B317" s="21" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C317" s="21"/>
       <c r="D317" s="21"/>
@@ -6713,7 +6725,7 @@
     <row r="318" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A318" s="2"/>
       <c r="B318" s="21" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C318" s="21"/>
       <c r="D318" s="21"/>
@@ -6722,7 +6734,7 @@
     <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A319" s="2"/>
       <c r="B319" s="21" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C319" s="21"/>
       <c r="D319" s="21"/>
@@ -6731,7 +6743,7 @@
     <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A320" s="2"/>
       <c r="B320" s="21" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C320" s="21" t="s">
         <v>22</v>
@@ -6742,7 +6754,7 @@
     <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="2"/>
       <c r="B321" s="21" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C321" s="21" t="s">
         <v>42</v>
@@ -6753,10 +6765,10 @@
     <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A322" s="2"/>
       <c r="B322" s="21" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C322" s="21" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D322" s="21"/>
       <c r="E322" s="11"/>
@@ -6764,7 +6776,7 @@
     <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A323" s="2"/>
       <c r="B323" s="21" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="C323" s="21" t="s">
         <v>51</v>
@@ -6775,16 +6787,16 @@
     <row r="324" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A324" s="2"/>
       <c r="B324" s="21" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C324" s="21" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D324" s="21" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="E324" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6797,7 +6809,7 @@
     <row r="326" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="6"/>
       <c r="B326" s="22" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C326" s="23"/>
       <c r="D326" s="23"/>
@@ -6815,7 +6827,7 @@
     <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A328" s="2"/>
       <c r="B328" s="21" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C328" s="21"/>
       <c r="D328" s="21"/>
@@ -6824,22 +6836,22 @@
     <row r="329" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A329" s="2"/>
       <c r="B329" s="21" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C329" s="21" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D329" s="21" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="E329" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A330" s="2"/>
       <c r="B330" s="21" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C330" s="21"/>
       <c r="D330" s="21"/>
@@ -6848,7 +6860,7 @@
     <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A331" s="2"/>
       <c r="B331" s="21" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C331" s="21"/>
       <c r="D331" s="21"/>
@@ -6857,16 +6869,16 @@
     <row r="332" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A332" s="2"/>
       <c r="B332" s="21" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="C332" s="21" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="D332" s="21" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="E332" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6879,7 +6891,7 @@
     <row r="334" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A334" s="6"/>
       <c r="B334" s="22" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C334" s="23"/>
       <c r="D334" s="23"/>
@@ -6897,7 +6909,7 @@
     <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A336" s="2"/>
       <c r="B336" s="21" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="C336" s="21"/>
       <c r="D336" s="21"/>
@@ -6906,7 +6918,7 @@
     <row r="337" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A337" s="2"/>
       <c r="B337" s="21" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C337" s="21"/>
       <c r="D337" s="21"/>
@@ -6915,22 +6927,22 @@
     <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A338" s="2"/>
       <c r="B338" s="21" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C338" s="21" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D338" s="21" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="E338" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A339" s="2"/>
       <c r="B339" s="21" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C339" s="21"/>
       <c r="D339" s="21"/>
@@ -6939,7 +6951,7 @@
     <row r="340" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A340" s="2"/>
       <c r="B340" s="21" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C340" s="21"/>
       <c r="D340" s="21"/>
@@ -6948,7 +6960,7 @@
     <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A341" s="2"/>
       <c r="B341" s="21" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C341" s="21"/>
       <c r="D341" s="21"/>
@@ -6957,40 +6969,40 @@
     <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A342" s="2"/>
       <c r="B342" s="21" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C342" s="21" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D342" s="21" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="E342" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A343" s="2"/>
       <c r="B343" s="21" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C343" s="21" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D343" s="21" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="E343" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="344" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="2"/>
       <c r="B344" s="21" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C344" s="21" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="D344" s="21"/>
       <c r="E344" s="11"/>
@@ -6998,31 +7010,31 @@
     <row r="345" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="2"/>
       <c r="B345" s="21" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C345" s="21" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D345" s="21" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="E345" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="346" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A346" s="2"/>
       <c r="B346" s="21" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C346" s="21" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="D346" s="21" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E346" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7035,7 +7047,7 @@
     <row r="348" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A348" s="26"/>
       <c r="B348" s="22" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C348" s="23"/>
       <c r="D348" s="23"/>
@@ -7053,7 +7065,7 @@
     <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A350" s="2"/>
       <c r="B350" s="21" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="C350" s="21"/>
       <c r="D350" s="21"/>
@@ -7062,22 +7074,22 @@
     <row r="351" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A351" s="2"/>
       <c r="B351" s="21" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C351" s="21" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D351" s="21" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="E351" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A352" s="2"/>
       <c r="B352" s="21" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="C352" s="21"/>
       <c r="D352" s="21"/>
@@ -7086,7 +7098,7 @@
     <row r="353" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A353" s="2"/>
       <c r="B353" s="21" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="C353" s="21"/>
       <c r="D353" s="21"/>
@@ -7095,7 +7107,7 @@
     <row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A354" s="2"/>
       <c r="B354" s="21" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C354" s="21"/>
       <c r="D354" s="21"/>
@@ -7104,10 +7116,10 @@
     <row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A355" s="2"/>
       <c r="B355" s="21" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C355" s="21" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D355" s="21"/>
       <c r="E355" s="11"/>
@@ -7115,10 +7127,10 @@
     <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A356" s="2"/>
       <c r="B356" s="21" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="C356" s="21" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D356" s="21"/>
       <c r="E356" s="11"/>
@@ -7126,10 +7138,10 @@
     <row r="357" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A357" s="2"/>
       <c r="B357" s="21" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C357" s="21" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="D357" s="21"/>
       <c r="E357" s="11"/>
@@ -7137,10 +7149,10 @@
     <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="2"/>
       <c r="B358" s="21" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="C358" s="21" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D358" s="21"/>
       <c r="E358" s="11"/>
@@ -7148,16 +7160,16 @@
     <row r="359" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A359" s="2"/>
       <c r="B359" s="21" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="C359" s="21" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="D359" s="21" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="E359" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7170,7 +7182,7 @@
     <row r="361" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="6"/>
       <c r="B361" s="22" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="C361" s="23"/>
       <c r="D361" s="23"/>
@@ -7188,7 +7200,7 @@
     <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A363" s="2"/>
       <c r="B363" s="21" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C363" s="21"/>
       <c r="D363" s="21"/>
@@ -7197,22 +7209,22 @@
     <row r="364" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A364" s="2"/>
       <c r="B364" s="21" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="C364" s="21" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D364" s="21" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="E364" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="2"/>
       <c r="B365" s="21" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C365" s="21"/>
       <c r="D365" s="21"/>
@@ -7221,7 +7233,7 @@
     <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A366" s="2"/>
       <c r="B366" s="21" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C366" s="21"/>
       <c r="D366" s="21"/>
@@ -7230,16 +7242,16 @@
     <row r="367" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="2"/>
       <c r="B367" s="21" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C367" s="21" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="D367" s="21" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="E367" s="11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="368" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7252,7 +7264,7 @@
     <row r="369" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A369" s="28"/>
       <c r="B369" s="29" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="C369" s="30"/>
       <c r="D369" s="30"/>
@@ -7270,7 +7282,7 @@
     <row r="371" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="2"/>
       <c r="B371" s="21" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="C371" s="21"/>
       <c r="D371" s="21"/>
@@ -7279,7 +7291,7 @@
     <row r="372" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="2"/>
       <c r="B372" s="21" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="C372" s="21"/>
       <c r="D372" s="21"/>
@@ -7288,10 +7300,10 @@
     <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="2"/>
       <c r="B373" s="21" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C373" s="21" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D373" s="21"/>
       <c r="E373" s="11"/>
@@ -7299,7 +7311,7 @@
     <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="2"/>
       <c r="B374" s="21" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C374" s="21"/>
       <c r="D374" s="21"/>
@@ -7308,7 +7320,7 @@
     <row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A375" s="2"/>
       <c r="B375" s="21" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C375" s="21"/>
       <c r="D375" s="21"/>
@@ -7317,7 +7329,7 @@
     <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="2"/>
       <c r="B376" s="21" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C376" s="21"/>
       <c r="D376" s="21"/>
@@ -7326,7 +7338,7 @@
     <row r="377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A377" s="2"/>
       <c r="B377" s="21" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="C377" s="21"/>
       <c r="D377" s="21"/>
@@ -7335,7 +7347,7 @@
     <row r="378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A378" s="2"/>
       <c r="B378" s="21" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="C378" s="21"/>
       <c r="D378" s="21"/>
@@ -7344,7 +7356,7 @@
     <row r="379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A379" s="2"/>
       <c r="B379" s="21" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C379" s="21"/>
       <c r="D379" s="21"/>
@@ -7353,7 +7365,7 @@
     <row r="380" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A380" s="2"/>
       <c r="B380" s="21" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="C380" s="21" t="s">
         <v>140</v>
@@ -7364,16 +7376,16 @@
     <row r="381" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="2"/>
       <c r="B381" s="21" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="C381" s="21" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="D381" s="21" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="E381" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7385,10 +7397,10 @@
     </row>
     <row r="383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A383" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B383" s="21" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C383" s="21"/>
       <c r="D383" s="21"/>
@@ -7397,7 +7409,7 @@
     <row r="384" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A384" s="2"/>
       <c r="B384" s="21" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="C384" s="21"/>
       <c r="D384" s="21"/>
@@ -7406,7 +7418,7 @@
     <row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="2"/>
       <c r="B385" s="21" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="C385" s="21"/>
       <c r="D385" s="21"/>
@@ -7415,7 +7427,7 @@
     <row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="2"/>
       <c r="B386" s="21" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="C386" s="21"/>
       <c r="D386" s="21"/>
@@ -7424,7 +7436,7 @@
     <row r="387" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="2"/>
       <c r="B387" s="21" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="C387" s="21"/>
       <c r="D387" s="21"/>
@@ -7433,22 +7445,22 @@
     <row r="388" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="2"/>
       <c r="B388" s="21" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="C388" s="21" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D388" s="21" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E388" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="2"/>
       <c r="B389" s="21" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="C389" s="21"/>
       <c r="D389" s="21"/>
@@ -7457,7 +7469,7 @@
     <row r="390" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A390" s="2"/>
       <c r="B390" s="21" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="C390" s="21"/>
       <c r="D390" s="21"/>
@@ -7466,7 +7478,7 @@
     <row r="391" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A391" s="2"/>
       <c r="B391" s="21" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C391" s="21"/>
       <c r="D391" s="21"/>
@@ -7475,22 +7487,22 @@
     <row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="2"/>
       <c r="B392" s="21" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="C392" s="21" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D392" s="21" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="E392" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="2"/>
       <c r="B393" s="21" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="C393" s="21"/>
       <c r="D393" s="21"/>
@@ -7506,7 +7518,7 @@
     <row r="395" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A395" s="6"/>
       <c r="B395" s="22" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="C395" s="23"/>
       <c r="D395" s="23"/>
@@ -7524,7 +7536,7 @@
     <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="2"/>
       <c r="B397" s="21" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="C397" s="21"/>
       <c r="D397" s="21"/>
@@ -7533,22 +7545,22 @@
     <row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="2"/>
       <c r="B398" s="21" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="C398" s="21" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D398" s="21" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="E398" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="399" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A399" s="2"/>
       <c r="B399" s="21" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="C399" s="21"/>
       <c r="D399" s="21"/>
@@ -7557,7 +7569,7 @@
     <row r="400" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A400" s="2"/>
       <c r="B400" s="21" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="C400" s="21"/>
       <c r="D400" s="21"/>
@@ -7566,7 +7578,7 @@
     <row r="401" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A401" s="2"/>
       <c r="B401" s="21" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="C401" s="21"/>
       <c r="D401" s="21"/>
@@ -7575,7 +7587,7 @@
     <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="2"/>
       <c r="B402" s="21" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="C402" s="21"/>
       <c r="D402" s="21"/>
@@ -7584,7 +7596,7 @@
     <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A403" s="2"/>
       <c r="B403" s="21" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="C403" s="21"/>
       <c r="D403" s="21"/>
@@ -7593,7 +7605,7 @@
     <row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A404" s="2"/>
       <c r="B404" s="21" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="C404" s="21"/>
       <c r="D404" s="21"/>
@@ -7602,7 +7614,7 @@
     <row r="405" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A405" s="2"/>
       <c r="B405" s="21" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="C405" s="21" t="s">
         <v>140</v>
@@ -7614,16 +7626,16 @@
     <row r="406" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A406" s="2"/>
       <c r="B406" s="21" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C406" s="21" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D406" s="21" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="E406" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7635,10 +7647,10 @@
     </row>
     <row r="408" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A408" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B408" s="21" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="C408" s="21"/>
       <c r="D408" s="21"/>
@@ -7647,7 +7659,7 @@
     <row r="409" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A409" s="2"/>
       <c r="B409" s="21" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C409" s="21"/>
       <c r="D409" s="21"/>
@@ -7656,10 +7668,10 @@
     <row r="410" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="2"/>
       <c r="B410" s="21" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="C410" s="21" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D410" s="21"/>
       <c r="E410" s="11"/>
@@ -7667,7 +7679,7 @@
     <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="2"/>
       <c r="B411" s="21" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="C411" s="21"/>
       <c r="D411" s="21"/>
@@ -7676,7 +7688,7 @@
     <row r="412" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="2"/>
       <c r="B412" s="21" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C412" s="21"/>
       <c r="D412" s="21"/>
@@ -7685,7 +7697,7 @@
     <row r="413" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A413" s="2"/>
       <c r="B413" s="21" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="C413" s="21"/>
       <c r="D413" s="21"/>
@@ -7694,10 +7706,10 @@
     <row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A414" s="2"/>
       <c r="B414" s="21" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C414" s="21" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D414" s="21"/>
       <c r="E414" s="11"/>
@@ -7705,7 +7717,7 @@
     <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="2"/>
       <c r="B415" s="21" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="C415" s="21"/>
       <c r="D415" s="21"/>
@@ -7714,7 +7726,7 @@
     <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="2"/>
       <c r="B416" s="21" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="C416" s="21"/>
       <c r="D416" s="21"/>
@@ -7723,7 +7735,7 @@
     <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="2"/>
       <c r="B417" s="21" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="C417" s="21"/>
       <c r="D417" s="21"/>
@@ -7732,7 +7744,7 @@
     <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="2"/>
       <c r="B418" s="21" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="C418" s="21"/>
       <c r="D418" s="21"/>
@@ -7741,7 +7753,7 @@
     <row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A419" s="2"/>
       <c r="B419" s="21" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="C419" s="21"/>
       <c r="D419" s="21"/>
@@ -7750,7 +7762,7 @@
     <row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A420" s="2"/>
       <c r="B420" s="21" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C420" s="21"/>
       <c r="D420" s="21"/>
@@ -7759,7 +7771,7 @@
     <row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A421" s="2"/>
       <c r="B421" s="21" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="C421" s="21"/>
       <c r="D421" s="21"/>
@@ -7768,22 +7780,22 @@
     <row r="422" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A422" s="2"/>
       <c r="B422" s="21" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="C422" s="21" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D422" s="21" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="E422" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="423" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A423" s="2"/>
       <c r="B423" s="21" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C423" s="21"/>
       <c r="D423" s="21"/>
@@ -7792,7 +7804,7 @@
     <row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A424" s="2"/>
       <c r="B424" s="21" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C424" s="21"/>
       <c r="D424" s="21"/>
@@ -7801,7 +7813,7 @@
     <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="2"/>
       <c r="B425" s="21" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="C425" s="21"/>
       <c r="D425" s="21"/>
@@ -7810,7 +7822,7 @@
     <row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A426" s="2"/>
       <c r="B426" s="21" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="C426" s="21"/>
       <c r="D426" s="21"/>
@@ -7819,7 +7831,7 @@
     <row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A427" s="2"/>
       <c r="B427" s="21" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="C427" s="21"/>
       <c r="D427" s="21"/>
@@ -7828,7 +7840,7 @@
     <row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A428" s="2"/>
       <c r="B428" s="21" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="C428" s="21"/>
       <c r="D428" s="21"/>
@@ -7837,7 +7849,7 @@
     <row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A429" s="2"/>
       <c r="B429" s="21" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C429" s="21"/>
       <c r="D429" s="21"/>
@@ -7846,28 +7858,28 @@
     <row r="430" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A430" s="2"/>
       <c r="B430" s="21" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C430" s="21" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="D430" s="21" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="E430" s="11" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="F430" s="18" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="G430" s="18" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="2"/>
       <c r="B431" s="21" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="C431" s="21"/>
       <c r="D431" s="21"/>
@@ -7876,7 +7888,7 @@
     <row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A432" s="2"/>
       <c r="B432" s="21" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="C432" s="21"/>
       <c r="D432" s="21"/>
@@ -7885,7 +7897,7 @@
     <row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A433" s="2"/>
       <c r="B433" s="21" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="C433" s="21"/>
       <c r="D433" s="21"/>
@@ -7894,7 +7906,7 @@
     <row r="434" customFormat="false" ht="36.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A434" s="2"/>
       <c r="B434" s="21" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="C434" s="21"/>
       <c r="D434" s="21"/>
@@ -7903,23 +7915,23 @@
     <row r="435" customFormat="false" ht="67.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A435" s="2"/>
       <c r="B435" s="21" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="C435" s="21" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="D435" s="21" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="E435" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F435" s="21"/>
     </row>
     <row r="436" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A436" s="2"/>
       <c r="B436" s="21" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="C436" s="21"/>
       <c r="D436" s="21"/>
@@ -7928,7 +7940,7 @@
     <row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A437" s="2"/>
       <c r="B437" s="21" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="C437" s="21"/>
       <c r="D437" s="21"/>
@@ -7937,35 +7949,35 @@
     <row r="438" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A438" s="2"/>
       <c r="B438" s="21" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C438" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D438" s="21"/>
       <c r="E438" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="439" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A439" s="2"/>
       <c r="B439" s="21" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C439" s="21" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D439" s="21" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="E439" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A440" s="2"/>
       <c r="B440" s="21" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="C440" s="21"/>
       <c r="D440" s="21"/>
@@ -7974,7 +7986,7 @@
     <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A441" s="2"/>
       <c r="B441" s="21" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="C441" s="21"/>
       <c r="D441" s="21"/>
@@ -7983,22 +7995,22 @@
     <row r="442" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A442" s="2"/>
       <c r="B442" s="21" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C442" s="21" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D442" s="21" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E442" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A443" s="2"/>
       <c r="B443" s="21" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="C443" s="21"/>
       <c r="D443" s="21"/>
@@ -8007,7 +8019,7 @@
     <row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A444" s="2"/>
       <c r="B444" s="21" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="C444" s="21"/>
       <c r="D444" s="21"/>
@@ -8016,22 +8028,22 @@
     <row r="445" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="2"/>
       <c r="B445" s="21" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="C445" s="21" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D445" s="21" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="E445" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="2"/>
       <c r="B446" s="21" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="C446" s="21"/>
       <c r="D446" s="21"/>
@@ -8046,10 +8058,10 @@
     </row>
     <row r="448" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A448" s="2" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="B448" s="21" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="C448" s="21"/>
       <c r="D448" s="21"/>
@@ -8058,22 +8070,22 @@
     <row r="449" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="2"/>
       <c r="B449" s="21" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C449" s="21" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D449" s="21" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="E449" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A450" s="2"/>
       <c r="B450" s="21" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C450" s="21"/>
       <c r="D450" s="21"/>
@@ -8089,7 +8101,7 @@
     <row r="452" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A452" s="6"/>
       <c r="B452" s="22" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="C452" s="23"/>
       <c r="D452" s="23"/>
@@ -8106,7 +8118,7 @@
     <row r="454" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A454" s="2"/>
       <c r="B454" s="21" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="C454" s="21"/>
       <c r="D454" s="21"/>
@@ -8115,7 +8127,7 @@
     <row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A455" s="2"/>
       <c r="B455" s="21" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C455" s="21"/>
       <c r="D455" s="21"/>
@@ -8124,7 +8136,7 @@
     <row r="456" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A456" s="2"/>
       <c r="B456" s="21" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="C456" s="21"/>
       <c r="D456" s="21"/>
@@ -8133,7 +8145,7 @@
     <row r="457" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A457" s="2"/>
       <c r="B457" s="21" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C457" s="21"/>
       <c r="D457" s="21"/>
@@ -8142,16 +8154,16 @@
     <row r="458" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A458" s="2"/>
       <c r="B458" s="21" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="C458" s="21" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D458" s="21" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E458" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8164,7 +8176,7 @@
     <row r="460" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A460" s="6"/>
       <c r="B460" s="22" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="C460" s="23"/>
       <c r="D460" s="23"/>
@@ -8181,7 +8193,7 @@
     <row r="462" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A462" s="2"/>
       <c r="B462" s="21" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="C462" s="21"/>
       <c r="D462" s="21"/>
@@ -8190,7 +8202,7 @@
     <row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A463" s="2"/>
       <c r="B463" s="21" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="C463" s="21"/>
       <c r="D463" s="21"/>
@@ -8199,10 +8211,10 @@
     <row r="464" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A464" s="2"/>
       <c r="B464" s="21" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="C464" s="21" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D464" s="21"/>
       <c r="E464" s="11"/>
@@ -8210,10 +8222,10 @@
     <row r="465" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="2"/>
       <c r="B465" s="21" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="C465" s="21" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="D465" s="21"/>
       <c r="E465" s="11"/>
@@ -8221,10 +8233,10 @@
     <row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A466" s="2"/>
       <c r="B466" s="21" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="C466" s="21" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D466" s="21"/>
       <c r="E466" s="11"/>
@@ -8232,13 +8244,13 @@
     <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A467" s="2"/>
       <c r="B467" s="21" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C467" s="21" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="D467" s="21" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E467" s="11" t="s">
         <v>24</v>
@@ -8247,22 +8259,22 @@
     <row r="468" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A468" s="2"/>
       <c r="B468" s="21" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="C468" s="21" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="D468" s="21" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="E468" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="469" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A469" s="2"/>
       <c r="B469" s="21" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="C469" s="21"/>
       <c r="D469" s="21"/>
@@ -8278,17 +8290,17 @@
     <row r="471" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A471" s="6"/>
       <c r="B471" s="22" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C471" s="23"/>
       <c r="D471" s="23" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="E471" s="23" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="F471" s="18" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8303,7 +8315,7 @@
     <row r="473" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A473" s="2"/>
       <c r="B473" s="21" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="C473" s="21"/>
       <c r="D473" s="21"/>
@@ -8312,25 +8324,25 @@
     <row r="474" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A474" s="2"/>
       <c r="B474" s="21" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="C474" s="21" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D474" s="21" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E474" s="11" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="F474" s="18" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="475" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A475" s="2"/>
       <c r="B475" s="21" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="C475" s="21"/>
       <c r="D475" s="21"/>
@@ -8339,7 +8351,7 @@
     <row r="476" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A476" s="2"/>
       <c r="B476" s="21" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="C476" s="21"/>
       <c r="D476" s="21"/>
@@ -8348,7 +8360,7 @@
     <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A477" s="2"/>
       <c r="B477" s="21" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="C477" s="21"/>
       <c r="D477" s="21"/>
@@ -8357,10 +8369,10 @@
     <row r="478" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A478" s="2"/>
       <c r="B478" s="21" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="C478" s="21" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="D478" s="21"/>
       <c r="E478" s="11"/>
@@ -8368,16 +8380,16 @@
     <row r="479" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A479" s="2"/>
       <c r="B479" s="21" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="C479" s="21" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="D479" s="21" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="E479" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8389,10 +8401,10 @@
     </row>
     <row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A481" s="2" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="B481" s="21" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="C481" s="21"/>
       <c r="D481" s="21"/>
@@ -8401,7 +8413,7 @@
     <row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A482" s="2"/>
       <c r="B482" s="21" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C482" s="21"/>
       <c r="D482" s="21"/>
@@ -8417,7 +8429,7 @@
     <row r="484" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A484" s="2"/>
       <c r="B484" s="21" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="C484" s="21"/>
       <c r="D484" s="21"/>
@@ -8426,7 +8438,7 @@
     <row r="485" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A485" s="2"/>
       <c r="B485" s="21" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="C485" s="21"/>
       <c r="D485" s="21"/>
@@ -8442,14 +8454,14 @@
     <row r="487" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A487" s="6"/>
       <c r="B487" s="22" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="C487" s="23"/>
       <c r="D487" s="23" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="E487" s="8" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8464,7 +8476,7 @@
     <row r="489" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A489" s="2"/>
       <c r="B489" s="21" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="C489" s="21"/>
       <c r="D489" s="21"/>
@@ -8473,35 +8485,35 @@
     <row r="490" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A490" s="2"/>
       <c r="B490" s="21" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="C490" s="21" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="D490" s="21" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E490" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="491" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A491" s="2"/>
       <c r="B491" s="21" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="C491" s="21"/>
       <c r="D491" s="21" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="E491" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="492" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A492" s="2"/>
       <c r="B492" s="21" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C492" s="21"/>
       <c r="D492" s="21"/>
@@ -8510,25 +8522,25 @@
     <row r="493" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A493" s="2"/>
       <c r="B493" s="21" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="C493" s="21" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D493" s="21" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E493" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F493" s="18" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
     </row>
     <row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A494" s="2"/>
       <c r="B494" s="21" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="C494" s="21"/>
       <c r="D494" s="21"/>
@@ -8537,7 +8549,7 @@
     <row r="495" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A495" s="2"/>
       <c r="B495" s="21" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="C495" s="21"/>
       <c r="D495" s="21"/>
@@ -8546,7 +8558,7 @@
     <row r="496" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A496" s="2"/>
       <c r="B496" s="21" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="C496" s="21"/>
       <c r="D496" s="21"/>
@@ -8555,7 +8567,7 @@
     <row r="497" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A497" s="2"/>
       <c r="B497" s="21" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="C497" s="21"/>
       <c r="D497" s="21"/>
@@ -8564,7 +8576,7 @@
     <row r="498" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A498" s="2"/>
       <c r="B498" s="21" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="C498" s="21"/>
       <c r="D498" s="21"/>
@@ -8573,7 +8585,7 @@
     <row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A499" s="2"/>
       <c r="B499" s="21" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C499" s="21"/>
       <c r="D499" s="21"/>
@@ -8582,7 +8594,7 @@
     <row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A500" s="2"/>
       <c r="B500" s="21" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="C500" s="21"/>
       <c r="D500" s="21"/>
@@ -8591,31 +8603,31 @@
     <row r="501" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A501" s="2"/>
       <c r="B501" s="21" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="C501" s="21" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="D501" s="21" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="E501" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="502" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A502" s="2"/>
       <c r="B502" s="21" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="C502" s="21" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="D502" s="21" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="E502" s="11" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="503" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8627,10 +8639,10 @@
     </row>
     <row r="504" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A504" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B504" s="21" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="C504" s="21"/>
       <c r="D504" s="21"/>
@@ -8639,7 +8651,7 @@
     <row r="505" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A505" s="2"/>
       <c r="B505" s="21" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="C505" s="21"/>
       <c r="D505" s="21"/>
@@ -8648,7 +8660,7 @@
     <row r="506" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A506" s="2"/>
       <c r="B506" s="21" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="C506" s="21"/>
       <c r="D506" s="21"/>
@@ -8657,7 +8669,7 @@
     <row r="507" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A507" s="2"/>
       <c r="B507" s="21" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="C507" s="21"/>
       <c r="D507" s="21"/>
@@ -8666,22 +8678,22 @@
     <row r="508" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A508" s="2"/>
       <c r="B508" s="21" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="C508" s="21" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="D508" s="21" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="E508" s="11" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="509" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A509" s="2"/>
       <c r="B509" s="21" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="C509" s="21"/>
       <c r="D509" s="21"/>
@@ -8690,7 +8702,7 @@
     <row r="510" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A510" s="2"/>
       <c r="B510" s="21" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="C510" s="21"/>
       <c r="D510" s="21"/>
@@ -8699,7 +8711,7 @@
     <row r="511" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A511" s="2"/>
       <c r="B511" s="21" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="C511" s="21"/>
       <c r="D511" s="21"/>
@@ -8708,7 +8720,7 @@
     <row r="512" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A512" s="2"/>
       <c r="B512" s="21" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="C512" s="21"/>
       <c r="D512" s="21"/>
@@ -8717,10 +8729,10 @@
     <row r="513" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A513" s="2"/>
       <c r="B513" s="21" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="C513" s="21" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="D513" s="21"/>
       <c r="E513" s="11"/>
@@ -8728,7 +8740,7 @@
     <row r="514" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A514" s="2"/>
       <c r="B514" s="21" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="C514" s="21"/>
       <c r="D514" s="21"/>
@@ -8737,7 +8749,7 @@
     <row r="515" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A515" s="2"/>
       <c r="B515" s="21" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="C515" s="21"/>
       <c r="D515" s="21"/>
@@ -8746,7 +8758,7 @@
     <row r="516" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A516" s="2"/>
       <c r="B516" s="21" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="C516" s="21"/>
       <c r="D516" s="21"/>
@@ -8755,7 +8767,7 @@
     <row r="517" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A517" s="2"/>
       <c r="B517" s="21" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="C517" s="21"/>
       <c r="D517" s="21"/>
@@ -8764,7 +8776,7 @@
     <row r="518" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A518" s="2"/>
       <c r="B518" s="21" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="C518" s="21"/>
       <c r="D518" s="21"/>
@@ -8773,7 +8785,7 @@
     <row r="519" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A519" s="2"/>
       <c r="B519" s="21" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="C519" s="21"/>
       <c r="D519" s="21"/>
@@ -8782,37 +8794,37 @@
     <row r="520" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A520" s="2"/>
       <c r="B520" s="21" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="C520" s="21" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D520" s="21" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="E520" s="11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="521" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A521" s="2"/>
       <c r="B521" s="21" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="C521" s="21" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="D521" s="21" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="E521" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="522" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A522" s="2"/>
       <c r="B522" s="21" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="C522" s="21"/>
       <c r="D522" s="21"/>
@@ -8827,10 +8839,10 @@
     </row>
     <row r="524" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A524" s="2" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="B524" s="21" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="C524" s="21"/>
       <c r="D524" s="21"/>
@@ -8839,7 +8851,7 @@
     <row r="525" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A525" s="2"/>
       <c r="B525" s="21" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="C525" s="21"/>
       <c r="D525" s="21"/>
@@ -8848,7 +8860,7 @@
     <row r="526" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A526" s="2"/>
       <c r="B526" s="21" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="C526" s="21"/>
       <c r="D526" s="21"/>
@@ -8857,16 +8869,16 @@
     <row r="527" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A527" s="2"/>
       <c r="B527" s="21" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="C527" s="21" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="D527" s="21" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="E527" s="11" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="528" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8879,7 +8891,7 @@
     <row r="529" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A529" s="2"/>
       <c r="B529" s="21" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="C529" s="21"/>
       <c r="D529" s="21"/>
@@ -8888,7 +8900,7 @@
     <row r="530" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A530" s="32"/>
       <c r="B530" s="33" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="C530" s="33"/>
       <c r="D530" s="33"/>

</xml_diff>

<commit_message>
+7 diagramas de sequencia
</commit_message>
<xml_diff>
--- a/assets/responsabilidades.xlsx
+++ b/assets/responsabilidades.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="672">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="671">
   <si>
     <t xml:space="preserve">Use Case</t>
   </si>
@@ -1160,7 +1160,7 @@
     <t xml:space="preserve">Atualizar stock</t>
   </si>
   <si>
-    <t xml:space="preserve">atualizaEstadoStock(id : int, estado : EstadosStock) : void</t>
+    <t xml:space="preserve">atualizaEstadoStock(id : int, estado : EstadoStock) : void</t>
   </si>
   <si>
     <t xml:space="preserve"> (alterar o estado das entradas de stock para ‘PendenteDevolucao’)</t>
@@ -1234,10 +1234,7 @@
     <t xml:space="preserve">9.1.2 O sistema atualiza o estado das entradas de stock devolvidas para o estado ‘Devolvida ao Fornecedor’</t>
   </si>
   <si>
-    <t xml:space="preserve">alteraEstado_Stock_Devolvida(pecas: List(string)) : void</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(alterar o estado das entradas de stock para ‘Devolvida_ao_Fornecedor’)</t>
+    <t xml:space="preserve">(alterar o estado das entradas de stock para ‘Devolvida_ao_Fornecedor’)/Repetir para todas as entradas</t>
   </si>
   <si>
     <t xml:space="preserve">9.1.3 Retorna ao passo 10</t>
@@ -5600,7 +5597,7 @@
       <c r="D209" s="21"/>
       <c r="E209" s="11"/>
     </row>
-    <row r="210" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="2"/>
       <c r="B210" s="21" t="s">
         <v>294</v>
@@ -5609,19 +5606,19 @@
         <v>276</v>
       </c>
       <c r="D210" s="21" t="s">
-        <v>295</v>
+        <v>277</v>
       </c>
       <c r="E210" s="11" t="s">
         <v>176</v>
       </c>
       <c r="F210" s="19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="2"/>
       <c r="B211" s="21" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C211" s="21"/>
       <c r="D211" s="21"/>
@@ -5630,7 +5627,7 @@
     <row r="212" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="2"/>
       <c r="B212" s="21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C212" s="21"/>
       <c r="D212" s="21"/>
@@ -5639,25 +5636,25 @@
     <row r="213" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="2"/>
       <c r="B213" s="21" t="s">
+        <v>298</v>
+      </c>
+      <c r="C213" s="21" t="s">
         <v>299</v>
       </c>
-      <c r="C213" s="21" t="s">
+      <c r="D213" s="21" t="s">
         <v>300</v>
-      </c>
-      <c r="D213" s="21" t="s">
-        <v>301</v>
       </c>
       <c r="E213" s="11" t="s">
         <v>131</v>
       </c>
       <c r="F213" s="19" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="2"/>
       <c r="B214" s="21" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C214" s="21"/>
       <c r="D214" s="21"/>
@@ -5673,7 +5670,7 @@
     <row r="216" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="6"/>
       <c r="B216" s="22" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C216" s="23"/>
       <c r="D216" s="23"/>
@@ -5691,7 +5688,7 @@
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="2"/>
       <c r="B218" s="21" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C218" s="21"/>
       <c r="D218" s="21"/>
@@ -5703,10 +5700,10 @@
         <v>282</v>
       </c>
       <c r="C219" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="D219" s="21" t="s">
         <v>306</v>
-      </c>
-      <c r="D219" s="21" t="s">
-        <v>307</v>
       </c>
       <c r="E219" s="11" t="s">
         <v>176</v>
@@ -5715,7 +5712,7 @@
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="2"/>
       <c r="B220" s="21" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C220" s="21"/>
       <c r="D220" s="21"/>
@@ -5724,13 +5721,13 @@
     <row r="221" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="2"/>
       <c r="B221" s="21" t="s">
+        <v>308</v>
+      </c>
+      <c r="C221" s="21" t="s">
         <v>309</v>
       </c>
-      <c r="C221" s="21" t="s">
+      <c r="D221" s="24" t="s">
         <v>310</v>
-      </c>
-      <c r="D221" s="24" t="s">
-        <v>311</v>
       </c>
       <c r="E221" s="11" t="s">
         <v>176</v>
@@ -5739,7 +5736,7 @@
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="2"/>
       <c r="B222" s="21" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C222" s="21"/>
       <c r="D222" s="21"/>
@@ -5748,13 +5745,13 @@
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="2"/>
       <c r="B223" s="21" t="s">
+        <v>312</v>
+      </c>
+      <c r="C223" s="21" t="s">
         <v>313</v>
       </c>
-      <c r="C223" s="21" t="s">
+      <c r="D223" s="21" t="s">
         <v>314</v>
-      </c>
-      <c r="D223" s="21" t="s">
-        <v>315</v>
       </c>
       <c r="E223" s="11" t="s">
         <v>176</v>
@@ -5763,13 +5760,13 @@
     <row r="224" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="2"/>
       <c r="B224" s="21" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C224" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="D224" s="21" t="s">
         <v>300</v>
-      </c>
-      <c r="D224" s="21" t="s">
-        <v>301</v>
       </c>
       <c r="E224" s="11" t="s">
         <v>131</v>
@@ -5778,7 +5775,7 @@
     <row r="225" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="2"/>
       <c r="B225" s="21" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C225" s="21"/>
       <c r="D225" s="21"/>
@@ -5797,7 +5794,7 @@
     <row r="227" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="6"/>
       <c r="B227" s="22" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C227" s="23"/>
       <c r="D227" s="23"/>
@@ -5815,7 +5812,7 @@
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="2"/>
       <c r="B229" s="21" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C229" s="21"/>
       <c r="D229" s="21"/>
@@ -5824,7 +5821,7 @@
     <row r="230" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="2"/>
       <c r="B230" s="21" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C230" s="21"/>
       <c r="D230" s="21"/>
@@ -5833,7 +5830,7 @@
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="2"/>
       <c r="B231" s="21" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C231" s="21"/>
       <c r="D231" s="21"/>
@@ -5853,10 +5850,10 @@
     <row r="233" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="2"/>
       <c r="B233" s="21" t="s">
+        <v>321</v>
+      </c>
+      <c r="C233" s="21" t="s">
         <v>322</v>
-      </c>
-      <c r="C233" s="21" t="s">
-        <v>323</v>
       </c>
       <c r="D233" s="21"/>
       <c r="E233" s="11"/>
@@ -5864,13 +5861,13 @@
     <row r="234" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="2"/>
       <c r="B234" s="21" t="s">
+        <v>323</v>
+      </c>
+      <c r="C234" s="21" t="s">
         <v>324</v>
       </c>
-      <c r="C234" s="21" t="s">
+      <c r="D234" s="21" t="s">
         <v>325</v>
-      </c>
-      <c r="D234" s="21" t="s">
-        <v>326</v>
       </c>
       <c r="E234" s="11" t="s">
         <v>176</v>
@@ -5886,7 +5883,7 @@
     <row r="236" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="6"/>
       <c r="B236" s="22" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C236" s="23"/>
       <c r="D236" s="23"/>
@@ -5904,7 +5901,7 @@
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="2"/>
       <c r="B238" s="21" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C238" s="21"/>
       <c r="D238" s="21"/>
@@ -5913,13 +5910,13 @@
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="2"/>
       <c r="B239" s="21" t="s">
+        <v>328</v>
+      </c>
+      <c r="C239" s="21" t="s">
         <v>329</v>
       </c>
-      <c r="C239" s="21" t="s">
+      <c r="D239" s="21" t="s">
         <v>330</v>
-      </c>
-      <c r="D239" s="21" t="s">
-        <v>331</v>
       </c>
       <c r="E239" s="11" t="s">
         <v>176</v>
@@ -5928,7 +5925,7 @@
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="2"/>
       <c r="B240" s="21" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C240" s="21"/>
       <c r="D240" s="21"/>
@@ -5955,7 +5952,7 @@
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="2"/>
       <c r="B243" s="21" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C243" s="21" t="s">
         <v>22</v>
@@ -5966,10 +5963,10 @@
     <row r="244" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="2"/>
       <c r="B244" s="21" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C244" s="21" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D244" s="21"/>
       <c r="E244" s="11"/>
@@ -5977,13 +5974,13 @@
     <row r="245" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="2"/>
       <c r="B245" s="21" t="s">
+        <v>334</v>
+      </c>
+      <c r="C245" s="21" t="s">
         <v>335</v>
       </c>
-      <c r="C245" s="21" t="s">
+      <c r="D245" s="21" t="s">
         <v>336</v>
-      </c>
-      <c r="D245" s="21" t="s">
-        <v>337</v>
       </c>
       <c r="E245" s="11" t="s">
         <v>176</v>
@@ -5999,7 +5996,7 @@
     <row r="247" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="6"/>
       <c r="B247" s="22" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C247" s="23"/>
       <c r="D247" s="23"/>
@@ -6017,7 +6014,7 @@
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="2"/>
       <c r="B249" s="21" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C249" s="21"/>
       <c r="D249" s="21"/>
@@ -6026,13 +6023,13 @@
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="2"/>
       <c r="B250" s="21" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C250" s="21" t="s">
+        <v>329</v>
+      </c>
+      <c r="D250" s="21" t="s">
         <v>330</v>
-      </c>
-      <c r="D250" s="21" t="s">
-        <v>331</v>
       </c>
       <c r="E250" s="11" t="s">
         <v>176</v>
@@ -6041,7 +6038,7 @@
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="2"/>
       <c r="B251" s="21" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C251" s="21"/>
       <c r="D251" s="21"/>
@@ -6050,7 +6047,7 @@
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="2"/>
       <c r="B252" s="21" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C252" s="21"/>
       <c r="D252" s="21"/>
@@ -6059,13 +6056,13 @@
     <row r="253" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="2"/>
       <c r="B253" s="21" t="s">
+        <v>342</v>
+      </c>
+      <c r="C253" s="21" t="s">
         <v>343</v>
       </c>
-      <c r="C253" s="21" t="s">
+      <c r="D253" s="21" t="s">
         <v>344</v>
-      </c>
-      <c r="D253" s="21" t="s">
-        <v>345</v>
       </c>
       <c r="E253" s="11" t="s">
         <v>176</v>
@@ -6082,7 +6079,7 @@
     <row r="255" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="6"/>
       <c r="B255" s="22" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C255" s="23"/>
       <c r="D255" s="23"/>
@@ -6100,7 +6097,7 @@
     <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="2"/>
       <c r="B257" s="21" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C257" s="21"/>
       <c r="D257" s="21"/>
@@ -6109,7 +6106,7 @@
     <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="2"/>
       <c r="B258" s="21" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C258" s="21"/>
       <c r="D258" s="21"/>
@@ -6118,13 +6115,13 @@
     <row r="259" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="2"/>
       <c r="B259" s="21" t="s">
+        <v>348</v>
+      </c>
+      <c r="C259" s="21" t="s">
         <v>349</v>
       </c>
-      <c r="C259" s="21" t="s">
+      <c r="D259" s="24" t="s">
         <v>350</v>
-      </c>
-      <c r="D259" s="24" t="s">
-        <v>351</v>
       </c>
       <c r="E259" s="25" t="s">
         <v>176</v>
@@ -6133,13 +6130,13 @@
     <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="2"/>
       <c r="B260" s="21" t="s">
+        <v>351</v>
+      </c>
+      <c r="C260" s="21" t="s">
         <v>352</v>
       </c>
-      <c r="C260" s="21" t="s">
+      <c r="D260" s="21" t="s">
         <v>353</v>
-      </c>
-      <c r="D260" s="21" t="s">
-        <v>354</v>
       </c>
       <c r="E260" s="11" t="s">
         <v>176</v>
@@ -6148,7 +6145,7 @@
     <row r="261" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="2"/>
       <c r="B261" s="21" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C261" s="21"/>
       <c r="D261" s="21"/>
@@ -6157,7 +6154,7 @@
     <row r="262" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="2"/>
       <c r="B262" s="21" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C262" s="21"/>
       <c r="D262" s="21"/>
@@ -6166,7 +6163,7 @@
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="2"/>
       <c r="B263" s="21" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C263" s="21"/>
       <c r="D263" s="21"/>
@@ -6175,7 +6172,7 @@
     <row r="264" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="2"/>
       <c r="B264" s="21" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C264" s="21"/>
       <c r="D264" s="21"/>
@@ -6184,7 +6181,7 @@
     <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="2"/>
       <c r="B265" s="21" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C265" s="21"/>
       <c r="D265" s="21"/>
@@ -6193,10 +6190,10 @@
     <row r="266" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="2"/>
       <c r="B266" s="21" t="s">
+        <v>359</v>
+      </c>
+      <c r="C266" s="21" t="s">
         <v>360</v>
-      </c>
-      <c r="C266" s="21" t="s">
-        <v>361</v>
       </c>
       <c r="D266" s="21"/>
       <c r="E266" s="11"/>
@@ -6204,13 +6201,13 @@
     <row r="267" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="2"/>
       <c r="B267" s="21" t="s">
+        <v>361</v>
+      </c>
+      <c r="C267" s="21" t="s">
         <v>362</v>
       </c>
-      <c r="C267" s="21" t="s">
+      <c r="D267" s="21" t="s">
         <v>363</v>
-      </c>
-      <c r="D267" s="21" t="s">
-        <v>364</v>
       </c>
       <c r="E267" s="11" t="s">
         <v>176</v>
@@ -6226,7 +6223,7 @@
     <row r="269" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="6"/>
       <c r="B269" s="22" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C269" s="23"/>
       <c r="D269" s="23"/>
@@ -6244,7 +6241,7 @@
     <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="2"/>
       <c r="B271" s="21" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C271" s="21"/>
       <c r="D271" s="21"/>
@@ -6253,13 +6250,13 @@
     <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="2"/>
       <c r="B272" s="21" t="s">
+        <v>366</v>
+      </c>
+      <c r="C272" s="21" t="s">
         <v>367</v>
       </c>
-      <c r="C272" s="21" t="s">
+      <c r="D272" s="21" t="s">
         <v>368</v>
-      </c>
-      <c r="D272" s="21" t="s">
-        <v>369</v>
       </c>
       <c r="E272" s="11" t="s">
         <v>176</v>
@@ -6268,7 +6265,7 @@
     <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="2"/>
       <c r="B273" s="21" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C273" s="21"/>
       <c r="D273" s="21"/>
@@ -6277,13 +6274,13 @@
     <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="2"/>
       <c r="B274" s="21" t="s">
+        <v>370</v>
+      </c>
+      <c r="C274" s="21" t="s">
         <v>371</v>
       </c>
-      <c r="C274" s="21" t="s">
+      <c r="D274" s="21" t="s">
         <v>372</v>
-      </c>
-      <c r="D274" s="21" t="s">
-        <v>373</v>
       </c>
       <c r="E274" s="11" t="s">
         <v>176</v>
@@ -6292,7 +6289,7 @@
     <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="2"/>
       <c r="B275" s="21" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C275" s="21"/>
       <c r="D275" s="21"/>
@@ -6301,7 +6298,7 @@
     <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="2"/>
       <c r="B276" s="21" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C276" s="21"/>
       <c r="D276" s="21"/>
@@ -6310,7 +6307,7 @@
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="2"/>
       <c r="B277" s="21" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C277" s="21" t="s">
         <v>290</v>
@@ -6321,13 +6318,13 @@
     <row r="278" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="2"/>
       <c r="B278" s="21" t="s">
+        <v>376</v>
+      </c>
+      <c r="C278" s="21" t="s">
         <v>377</v>
       </c>
-      <c r="C278" s="21" t="s">
+      <c r="D278" s="21" t="s">
         <v>378</v>
-      </c>
-      <c r="D278" s="21" t="s">
-        <v>379</v>
       </c>
       <c r="E278" s="11" t="s">
         <v>176</v>
@@ -6345,7 +6342,7 @@
         <v>236</v>
       </c>
       <c r="B280" s="21" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C280" s="21"/>
       <c r="D280" s="21"/>
@@ -6354,7 +6351,7 @@
     <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="2"/>
       <c r="B281" s="21" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C281" s="21"/>
       <c r="D281" s="21"/>
@@ -6363,7 +6360,7 @@
     <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="2"/>
       <c r="B282" s="21" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C282" s="21"/>
       <c r="D282" s="21"/>
@@ -6372,10 +6369,10 @@
     <row r="283" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="2"/>
       <c r="B283" s="21" t="s">
+        <v>382</v>
+      </c>
+      <c r="C283" s="21" t="s">
         <v>383</v>
-      </c>
-      <c r="C283" s="21" t="s">
-        <v>384</v>
       </c>
       <c r="D283" s="21"/>
       <c r="E283" s="11"/>
@@ -6383,13 +6380,13 @@
     <row r="284" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="2"/>
       <c r="B284" s="21" t="s">
+        <v>384</v>
+      </c>
+      <c r="C284" s="21" t="s">
         <v>385</v>
       </c>
-      <c r="C284" s="21" t="s">
+      <c r="D284" s="21" t="s">
         <v>386</v>
-      </c>
-      <c r="D284" s="21" t="s">
-        <v>387</v>
       </c>
       <c r="E284" s="11" t="s">
         <v>176</v>
@@ -6398,7 +6395,7 @@
     <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="2"/>
       <c r="B285" s="21" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C285" s="21"/>
       <c r="D285" s="21"/>
@@ -6407,7 +6404,7 @@
     <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="2"/>
       <c r="B286" s="21" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C286" s="21"/>
       <c r="D286" s="21"/>
@@ -6416,7 +6413,7 @@
     <row r="287" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="2"/>
       <c r="B287" s="21" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C287" s="21"/>
       <c r="D287" s="21"/>
@@ -6425,7 +6422,7 @@
     <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="2"/>
       <c r="B288" s="21" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C288" s="21"/>
       <c r="D288" s="21"/>
@@ -6434,10 +6431,10 @@
     <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="2"/>
       <c r="B289" s="21" t="s">
+        <v>391</v>
+      </c>
+      <c r="C289" s="21" t="s">
         <v>392</v>
-      </c>
-      <c r="C289" s="21" t="s">
-        <v>393</v>
       </c>
       <c r="D289" s="21"/>
       <c r="E289" s="11"/>
@@ -6445,10 +6442,10 @@
     <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="2"/>
       <c r="B290" s="21" t="s">
+        <v>393</v>
+      </c>
+      <c r="C290" s="21" t="s">
         <v>394</v>
-      </c>
-      <c r="C290" s="21" t="s">
-        <v>395</v>
       </c>
       <c r="D290" s="21"/>
       <c r="E290" s="11"/>
@@ -6456,13 +6453,13 @@
     <row r="291" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="2"/>
       <c r="B291" s="21" t="s">
+        <v>395</v>
+      </c>
+      <c r="C291" s="21" t="s">
+        <v>385</v>
+      </c>
+      <c r="D291" s="21" t="s">
         <v>396</v>
-      </c>
-      <c r="C291" s="21" t="s">
-        <v>386</v>
-      </c>
-      <c r="D291" s="21" t="s">
-        <v>397</v>
       </c>
       <c r="E291" s="11" t="s">
         <v>176</v>
@@ -6471,7 +6468,7 @@
     <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="2"/>
       <c r="B292" s="21" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C292" s="21"/>
       <c r="D292" s="21"/>
@@ -6487,7 +6484,7 @@
     <row r="294" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A294" s="6"/>
       <c r="B294" s="22" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C294" s="23"/>
       <c r="D294" s="23"/>
@@ -6505,7 +6502,7 @@
     <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="2"/>
       <c r="B296" s="21" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C296" s="21"/>
       <c r="D296" s="21"/>
@@ -6514,7 +6511,7 @@
     <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A297" s="2"/>
       <c r="B297" s="21" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C297" s="21"/>
       <c r="D297" s="21"/>
@@ -6523,7 +6520,7 @@
     <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="2"/>
       <c r="B298" s="21" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C298" s="21"/>
       <c r="D298" s="21"/>
@@ -6532,7 +6529,7 @@
     <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="2"/>
       <c r="B299" s="21" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C299" s="21"/>
       <c r="D299" s="21"/>
@@ -6541,13 +6538,13 @@
     <row r="300" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A300" s="2"/>
       <c r="B300" s="21" t="s">
+        <v>402</v>
+      </c>
+      <c r="C300" s="21" t="s">
         <v>403</v>
       </c>
-      <c r="C300" s="21" t="s">
+      <c r="D300" s="21" t="s">
         <v>404</v>
-      </c>
-      <c r="D300" s="21" t="s">
-        <v>405</v>
       </c>
       <c r="E300" s="11" t="s">
         <v>176</v>
@@ -6563,7 +6560,7 @@
     <row r="302" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A302" s="6"/>
       <c r="B302" s="22" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C302" s="23"/>
       <c r="D302" s="23"/>
@@ -6581,7 +6578,7 @@
     <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A304" s="2"/>
       <c r="B304" s="21" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C304" s="21"/>
       <c r="D304" s="21"/>
@@ -6590,7 +6587,7 @@
     <row r="305" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="2"/>
       <c r="B305" s="21" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C305" s="21"/>
       <c r="D305" s="21"/>
@@ -6599,7 +6596,7 @@
     <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A306" s="2"/>
       <c r="B306" s="21" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C306" s="21"/>
       <c r="D306" s="21"/>
@@ -6619,7 +6616,7 @@
     <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A308" s="2"/>
       <c r="B308" s="21" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C308" s="21" t="s">
         <v>42</v>
@@ -6630,10 +6627,10 @@
     <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A309" s="2"/>
       <c r="B309" s="21" t="s">
+        <v>409</v>
+      </c>
+      <c r="C309" s="21" t="s">
         <v>410</v>
-      </c>
-      <c r="C309" s="21" t="s">
-        <v>411</v>
       </c>
       <c r="D309" s="21"/>
       <c r="E309" s="11"/>
@@ -6641,7 +6638,7 @@
     <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A310" s="2"/>
       <c r="B310" s="21" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C310" s="21" t="s">
         <v>51</v>
@@ -6652,16 +6649,16 @@
     <row r="311" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A311" s="2"/>
       <c r="B311" s="21" t="s">
+        <v>412</v>
+      </c>
+      <c r="C311" s="21" t="s">
         <v>413</v>
       </c>
-      <c r="C311" s="21" t="s">
+      <c r="D311" s="21" t="s">
         <v>414</v>
       </c>
-      <c r="D311" s="21" t="s">
+      <c r="E311" s="11" t="s">
         <v>415</v>
-      </c>
-      <c r="E311" s="11" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6674,7 +6671,7 @@
     <row r="313" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="6"/>
       <c r="B313" s="22" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C313" s="23"/>
       <c r="D313" s="23"/>
@@ -6692,7 +6689,7 @@
     <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A315" s="2"/>
       <c r="B315" s="21" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C315" s="21"/>
       <c r="D315" s="21"/>
@@ -6701,22 +6698,22 @@
     <row r="316" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A316" s="2"/>
       <c r="B316" s="21" t="s">
+        <v>418</v>
+      </c>
+      <c r="C316" s="21" t="s">
         <v>419</v>
       </c>
-      <c r="C316" s="21" t="s">
+      <c r="D316" s="21" t="s">
         <v>420</v>
       </c>
-      <c r="D316" s="21" t="s">
-        <v>421</v>
-      </c>
       <c r="E316" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A317" s="2"/>
       <c r="B317" s="21" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C317" s="21"/>
       <c r="D317" s="21"/>
@@ -6743,7 +6740,7 @@
     <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A320" s="2"/>
       <c r="B320" s="21" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C320" s="21" t="s">
         <v>22</v>
@@ -6754,7 +6751,7 @@
     <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="2"/>
       <c r="B321" s="21" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C321" s="21" t="s">
         <v>42</v>
@@ -6765,10 +6762,10 @@
     <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A322" s="2"/>
       <c r="B322" s="21" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C322" s="21" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="D322" s="21"/>
       <c r="E322" s="11"/>
@@ -6776,7 +6773,7 @@
     <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A323" s="2"/>
       <c r="B323" s="21" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C323" s="21" t="s">
         <v>51</v>
@@ -6787,16 +6784,16 @@
     <row r="324" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A324" s="2"/>
       <c r="B324" s="21" t="s">
+        <v>425</v>
+      </c>
+      <c r="C324" s="21" t="s">
         <v>426</v>
       </c>
-      <c r="C324" s="21" t="s">
+      <c r="D324" s="21" t="s">
         <v>427</v>
       </c>
-      <c r="D324" s="21" t="s">
-        <v>428</v>
-      </c>
       <c r="E324" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6809,7 +6806,7 @@
     <row r="326" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="6"/>
       <c r="B326" s="22" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C326" s="23"/>
       <c r="D326" s="23"/>
@@ -6827,7 +6824,7 @@
     <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A328" s="2"/>
       <c r="B328" s="21" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C328" s="21"/>
       <c r="D328" s="21"/>
@@ -6836,22 +6833,22 @@
     <row r="329" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A329" s="2"/>
       <c r="B329" s="21" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C329" s="21" t="s">
+        <v>419</v>
+      </c>
+      <c r="D329" s="21" t="s">
         <v>420</v>
       </c>
-      <c r="D329" s="21" t="s">
-        <v>421</v>
-      </c>
       <c r="E329" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A330" s="2"/>
       <c r="B330" s="21" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C330" s="21"/>
       <c r="D330" s="21"/>
@@ -6860,7 +6857,7 @@
     <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A331" s="2"/>
       <c r="B331" s="21" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C331" s="21"/>
       <c r="D331" s="21"/>
@@ -6869,16 +6866,16 @@
     <row r="332" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A332" s="2"/>
       <c r="B332" s="21" t="s">
+        <v>432</v>
+      </c>
+      <c r="C332" s="21" t="s">
         <v>433</v>
       </c>
-      <c r="C332" s="21" t="s">
+      <c r="D332" s="21" t="s">
         <v>434</v>
       </c>
-      <c r="D332" s="21" t="s">
-        <v>435</v>
-      </c>
       <c r="E332" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6891,7 +6888,7 @@
     <row r="334" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A334" s="6"/>
       <c r="B334" s="22" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C334" s="23"/>
       <c r="D334" s="23"/>
@@ -6909,7 +6906,7 @@
     <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A336" s="2"/>
       <c r="B336" s="21" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C336" s="21"/>
       <c r="D336" s="21"/>
@@ -6918,7 +6915,7 @@
     <row r="337" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A337" s="2"/>
       <c r="B337" s="21" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C337" s="21"/>
       <c r="D337" s="21"/>
@@ -6927,22 +6924,22 @@
     <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A338" s="2"/>
       <c r="B338" s="21" t="s">
+        <v>438</v>
+      </c>
+      <c r="C338" s="21" t="s">
         <v>439</v>
       </c>
-      <c r="C338" s="21" t="s">
+      <c r="D338" s="21" t="s">
         <v>440</v>
       </c>
-      <c r="D338" s="21" t="s">
-        <v>441</v>
-      </c>
       <c r="E338" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A339" s="2"/>
       <c r="B339" s="21" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C339" s="21"/>
       <c r="D339" s="21"/>
@@ -6951,7 +6948,7 @@
     <row r="340" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A340" s="2"/>
       <c r="B340" s="21" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C340" s="21"/>
       <c r="D340" s="21"/>
@@ -6960,7 +6957,7 @@
     <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A341" s="2"/>
       <c r="B341" s="21" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C341" s="21"/>
       <c r="D341" s="21"/>
@@ -6969,40 +6966,40 @@
     <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A342" s="2"/>
       <c r="B342" s="21" t="s">
+        <v>444</v>
+      </c>
+      <c r="C342" s="21" t="s">
         <v>445</v>
       </c>
-      <c r="C342" s="21" t="s">
+      <c r="D342" s="21" t="s">
         <v>446</v>
       </c>
-      <c r="D342" s="21" t="s">
-        <v>447</v>
-      </c>
       <c r="E342" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A343" s="2"/>
       <c r="B343" s="21" t="s">
+        <v>447</v>
+      </c>
+      <c r="C343" s="21" t="s">
         <v>448</v>
       </c>
-      <c r="C343" s="21" t="s">
+      <c r="D343" s="21" t="s">
         <v>449</v>
       </c>
-      <c r="D343" s="21" t="s">
-        <v>450</v>
-      </c>
       <c r="E343" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="344" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="2"/>
       <c r="B344" s="21" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C344" s="21" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D344" s="21"/>
       <c r="E344" s="11"/>
@@ -7010,31 +7007,31 @@
     <row r="345" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="2"/>
       <c r="B345" s="21" t="s">
+        <v>451</v>
+      </c>
+      <c r="C345" s="21" t="s">
         <v>452</v>
       </c>
-      <c r="C345" s="21" t="s">
+      <c r="D345" s="21" t="s">
         <v>453</v>
       </c>
-      <c r="D345" s="21" t="s">
-        <v>454</v>
-      </c>
       <c r="E345" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="346" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A346" s="2"/>
       <c r="B346" s="21" t="s">
+        <v>454</v>
+      </c>
+      <c r="C346" s="21" t="s">
         <v>455</v>
       </c>
-      <c r="C346" s="21" t="s">
+      <c r="D346" s="21" t="s">
         <v>456</v>
       </c>
-      <c r="D346" s="21" t="s">
-        <v>457</v>
-      </c>
       <c r="E346" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7047,7 +7044,7 @@
     <row r="348" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A348" s="26"/>
       <c r="B348" s="22" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C348" s="23"/>
       <c r="D348" s="23"/>
@@ -7065,7 +7062,7 @@
     <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A350" s="2"/>
       <c r="B350" s="21" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C350" s="21"/>
       <c r="D350" s="21"/>
@@ -7074,22 +7071,22 @@
     <row r="351" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A351" s="2"/>
       <c r="B351" s="21" t="s">
+        <v>459</v>
+      </c>
+      <c r="C351" s="21" t="s">
         <v>460</v>
       </c>
-      <c r="C351" s="21" t="s">
+      <c r="D351" s="21" t="s">
         <v>461</v>
       </c>
-      <c r="D351" s="21" t="s">
-        <v>462</v>
-      </c>
       <c r="E351" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A352" s="2"/>
       <c r="B352" s="21" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C352" s="21"/>
       <c r="D352" s="21"/>
@@ -7098,7 +7095,7 @@
     <row r="353" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A353" s="2"/>
       <c r="B353" s="21" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C353" s="21"/>
       <c r="D353" s="21"/>
@@ -7116,10 +7113,10 @@
     <row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A355" s="2"/>
       <c r="B355" s="21" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C355" s="21" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D355" s="21"/>
       <c r="E355" s="11"/>
@@ -7127,10 +7124,10 @@
     <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A356" s="2"/>
       <c r="B356" s="21" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C356" s="21" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D356" s="21"/>
       <c r="E356" s="11"/>
@@ -7138,10 +7135,10 @@
     <row r="357" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A357" s="2"/>
       <c r="B357" s="21" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C357" s="21" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D357" s="21"/>
       <c r="E357" s="11"/>
@@ -7149,10 +7146,10 @@
     <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="2"/>
       <c r="B358" s="21" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C358" s="21" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="D358" s="21"/>
       <c r="E358" s="11"/>
@@ -7160,16 +7157,16 @@
     <row r="359" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A359" s="2"/>
       <c r="B359" s="21" t="s">
+        <v>468</v>
+      </c>
+      <c r="C359" s="21" t="s">
         <v>469</v>
       </c>
-      <c r="C359" s="21" t="s">
+      <c r="D359" s="21" t="s">
         <v>470</v>
       </c>
-      <c r="D359" s="21" t="s">
-        <v>471</v>
-      </c>
       <c r="E359" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7182,7 +7179,7 @@
     <row r="361" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="6"/>
       <c r="B361" s="22" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C361" s="23"/>
       <c r="D361" s="23"/>
@@ -7200,7 +7197,7 @@
     <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A363" s="2"/>
       <c r="B363" s="21" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C363" s="21"/>
       <c r="D363" s="21"/>
@@ -7209,22 +7206,22 @@
     <row r="364" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A364" s="2"/>
       <c r="B364" s="21" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C364" s="21" t="s">
+        <v>460</v>
+      </c>
+      <c r="D364" s="21" t="s">
         <v>461</v>
       </c>
-      <c r="D364" s="21" t="s">
-        <v>462</v>
-      </c>
       <c r="E364" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="2"/>
       <c r="B365" s="21" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C365" s="21"/>
       <c r="D365" s="21"/>
@@ -7233,7 +7230,7 @@
     <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A366" s="2"/>
       <c r="B366" s="21" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C366" s="21"/>
       <c r="D366" s="21"/>
@@ -7242,16 +7239,16 @@
     <row r="367" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="2"/>
       <c r="B367" s="21" t="s">
+        <v>475</v>
+      </c>
+      <c r="C367" s="21" t="s">
         <v>476</v>
       </c>
-      <c r="C367" s="21" t="s">
+      <c r="D367" s="21" t="s">
         <v>477</v>
       </c>
-      <c r="D367" s="21" t="s">
-        <v>478</v>
-      </c>
       <c r="E367" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="368" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7264,7 +7261,7 @@
     <row r="369" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A369" s="28"/>
       <c r="B369" s="29" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C369" s="30"/>
       <c r="D369" s="30"/>
@@ -7282,7 +7279,7 @@
     <row r="371" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="2"/>
       <c r="B371" s="21" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C371" s="21"/>
       <c r="D371" s="21"/>
@@ -7291,7 +7288,7 @@
     <row r="372" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="2"/>
       <c r="B372" s="21" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C372" s="21"/>
       <c r="D372" s="21"/>
@@ -7300,10 +7297,10 @@
     <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="2"/>
       <c r="B373" s="21" t="s">
+        <v>438</v>
+      </c>
+      <c r="C373" s="21" t="s">
         <v>439</v>
-      </c>
-      <c r="C373" s="21" t="s">
-        <v>440</v>
       </c>
       <c r="D373" s="21"/>
       <c r="E373" s="11"/>
@@ -7311,7 +7308,7 @@
     <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="2"/>
       <c r="B374" s="21" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C374" s="21"/>
       <c r="D374" s="21"/>
@@ -7320,7 +7317,7 @@
     <row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A375" s="2"/>
       <c r="B375" s="21" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C375" s="21"/>
       <c r="D375" s="21"/>
@@ -7329,7 +7326,7 @@
     <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="2"/>
       <c r="B376" s="21" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C376" s="21"/>
       <c r="D376" s="21"/>
@@ -7338,7 +7335,7 @@
     <row r="377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A377" s="2"/>
       <c r="B377" s="21" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C377" s="21"/>
       <c r="D377" s="21"/>
@@ -7347,7 +7344,7 @@
     <row r="378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A378" s="2"/>
       <c r="B378" s="21" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C378" s="21"/>
       <c r="D378" s="21"/>
@@ -7356,7 +7353,7 @@
     <row r="379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A379" s="2"/>
       <c r="B379" s="21" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C379" s="21"/>
       <c r="D379" s="21"/>
@@ -7365,7 +7362,7 @@
     <row r="380" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A380" s="2"/>
       <c r="B380" s="21" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C380" s="21" t="s">
         <v>140</v>
@@ -7376,16 +7373,16 @@
     <row r="381" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="2"/>
       <c r="B381" s="21" t="s">
+        <v>487</v>
+      </c>
+      <c r="C381" s="21" t="s">
         <v>488</v>
       </c>
-      <c r="C381" s="21" t="s">
+      <c r="D381" s="21" t="s">
         <v>489</v>
       </c>
-      <c r="D381" s="21" t="s">
+      <c r="E381" s="11" t="s">
         <v>490</v>
-      </c>
-      <c r="E381" s="11" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7400,7 +7397,7 @@
         <v>236</v>
       </c>
       <c r="B383" s="21" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C383" s="21"/>
       <c r="D383" s="21"/>
@@ -7409,7 +7406,7 @@
     <row r="384" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A384" s="2"/>
       <c r="B384" s="21" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C384" s="21"/>
       <c r="D384" s="21"/>
@@ -7418,7 +7415,7 @@
     <row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="2"/>
       <c r="B385" s="21" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C385" s="21"/>
       <c r="D385" s="21"/>
@@ -7427,7 +7424,7 @@
     <row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="2"/>
       <c r="B386" s="21" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C386" s="21"/>
       <c r="D386" s="21"/>
@@ -7436,7 +7433,7 @@
     <row r="387" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="2"/>
       <c r="B387" s="21" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C387" s="21"/>
       <c r="D387" s="21"/>
@@ -7445,22 +7442,22 @@
     <row r="388" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="2"/>
       <c r="B388" s="21" t="s">
+        <v>496</v>
+      </c>
+      <c r="C388" s="21" t="s">
         <v>497</v>
       </c>
-      <c r="C388" s="21" t="s">
+      <c r="D388" s="21" t="s">
         <v>498</v>
       </c>
-      <c r="D388" s="21" t="s">
-        <v>499</v>
-      </c>
       <c r="E388" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="2"/>
       <c r="B389" s="21" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C389" s="21"/>
       <c r="D389" s="21"/>
@@ -7469,7 +7466,7 @@
     <row r="390" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A390" s="2"/>
       <c r="B390" s="21" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C390" s="21"/>
       <c r="D390" s="21"/>
@@ -7478,7 +7475,7 @@
     <row r="391" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A391" s="2"/>
       <c r="B391" s="21" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C391" s="21"/>
       <c r="D391" s="21"/>
@@ -7487,22 +7484,22 @@
     <row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="2"/>
       <c r="B392" s="21" t="s">
+        <v>502</v>
+      </c>
+      <c r="C392" s="21" t="s">
         <v>503</v>
       </c>
-      <c r="C392" s="21" t="s">
+      <c r="D392" s="21" t="s">
         <v>504</v>
       </c>
-      <c r="D392" s="21" t="s">
-        <v>505</v>
-      </c>
       <c r="E392" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="2"/>
       <c r="B393" s="21" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C393" s="21"/>
       <c r="D393" s="21"/>
@@ -7518,7 +7515,7 @@
     <row r="395" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A395" s="6"/>
       <c r="B395" s="22" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C395" s="23"/>
       <c r="D395" s="23"/>
@@ -7536,7 +7533,7 @@
     <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="2"/>
       <c r="B397" s="21" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C397" s="21"/>
       <c r="D397" s="21"/>
@@ -7545,22 +7542,22 @@
     <row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="2"/>
       <c r="B398" s="21" t="s">
+        <v>508</v>
+      </c>
+      <c r="C398" s="21" t="s">
         <v>509</v>
       </c>
-      <c r="C398" s="21" t="s">
+      <c r="D398" s="21" t="s">
         <v>510</v>
       </c>
-      <c r="D398" s="21" t="s">
-        <v>511</v>
-      </c>
       <c r="E398" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="399" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A399" s="2"/>
       <c r="B399" s="21" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C399" s="21"/>
       <c r="D399" s="21"/>
@@ -7569,7 +7566,7 @@
     <row r="400" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A400" s="2"/>
       <c r="B400" s="21" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C400" s="21"/>
       <c r="D400" s="21"/>
@@ -7578,7 +7575,7 @@
     <row r="401" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A401" s="2"/>
       <c r="B401" s="21" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="C401" s="21"/>
       <c r="D401" s="21"/>
@@ -7587,7 +7584,7 @@
     <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="2"/>
       <c r="B402" s="21" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C402" s="21"/>
       <c r="D402" s="21"/>
@@ -7596,7 +7593,7 @@
     <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A403" s="2"/>
       <c r="B403" s="21" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="C403" s="21"/>
       <c r="D403" s="21"/>
@@ -7605,7 +7602,7 @@
     <row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A404" s="2"/>
       <c r="B404" s="21" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C404" s="21"/>
       <c r="D404" s="21"/>
@@ -7614,7 +7611,7 @@
     <row r="405" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A405" s="2"/>
       <c r="B405" s="21" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="C405" s="21" t="s">
         <v>140</v>
@@ -7626,16 +7623,16 @@
     <row r="406" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A406" s="2"/>
       <c r="B406" s="21" t="s">
+        <v>518</v>
+      </c>
+      <c r="C406" s="21" t="s">
         <v>519</v>
       </c>
-      <c r="C406" s="21" t="s">
+      <c r="D406" s="21" t="s">
         <v>520</v>
       </c>
-      <c r="D406" s="21" t="s">
-        <v>521</v>
-      </c>
       <c r="E406" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7650,7 +7647,7 @@
         <v>236</v>
       </c>
       <c r="B408" s="21" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C408" s="21"/>
       <c r="D408" s="21"/>
@@ -7659,7 +7656,7 @@
     <row r="409" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A409" s="2"/>
       <c r="B409" s="21" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C409" s="21"/>
       <c r="D409" s="21"/>
@@ -7668,10 +7665,10 @@
     <row r="410" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="2"/>
       <c r="B410" s="21" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="C410" s="21" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="D410" s="21"/>
       <c r="E410" s="11"/>
@@ -7679,7 +7676,7 @@
     <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="2"/>
       <c r="B411" s="21" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C411" s="21"/>
       <c r="D411" s="21"/>
@@ -7688,7 +7685,7 @@
     <row r="412" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="2"/>
       <c r="B412" s="21" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="C412" s="21"/>
       <c r="D412" s="21"/>
@@ -7697,7 +7694,7 @@
     <row r="413" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A413" s="2"/>
       <c r="B413" s="21" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C413" s="21"/>
       <c r="D413" s="21"/>
@@ -7706,10 +7703,10 @@
     <row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A414" s="2"/>
       <c r="B414" s="21" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="C414" s="21" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D414" s="21"/>
       <c r="E414" s="11"/>
@@ -7717,7 +7714,7 @@
     <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="2"/>
       <c r="B415" s="21" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C415" s="21"/>
       <c r="D415" s="21"/>
@@ -7726,7 +7723,7 @@
     <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="2"/>
       <c r="B416" s="21" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C416" s="21"/>
       <c r="D416" s="21"/>
@@ -7735,7 +7732,7 @@
     <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="2"/>
       <c r="B417" s="21" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="C417" s="21"/>
       <c r="D417" s="21"/>
@@ -7744,7 +7741,7 @@
     <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="2"/>
       <c r="B418" s="21" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C418" s="21"/>
       <c r="D418" s="21"/>
@@ -7753,7 +7750,7 @@
     <row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A419" s="2"/>
       <c r="B419" s="21" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="C419" s="21"/>
       <c r="D419" s="21"/>
@@ -7762,7 +7759,7 @@
     <row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A420" s="2"/>
       <c r="B420" s="21" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C420" s="21"/>
       <c r="D420" s="21"/>
@@ -7771,7 +7768,7 @@
     <row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A421" s="2"/>
       <c r="B421" s="21" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="C421" s="21"/>
       <c r="D421" s="21"/>
@@ -7780,22 +7777,22 @@
     <row r="422" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A422" s="2"/>
       <c r="B422" s="21" t="s">
+        <v>535</v>
+      </c>
+      <c r="C422" s="21" t="s">
         <v>536</v>
       </c>
-      <c r="C422" s="21" t="s">
+      <c r="D422" s="21" t="s">
         <v>537</v>
       </c>
-      <c r="D422" s="21" t="s">
-        <v>538</v>
-      </c>
       <c r="E422" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="423" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A423" s="2"/>
       <c r="B423" s="21" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C423" s="21"/>
       <c r="D423" s="21"/>
@@ -7804,7 +7801,7 @@
     <row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A424" s="2"/>
       <c r="B424" s="21" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="C424" s="21"/>
       <c r="D424" s="21"/>
@@ -7813,7 +7810,7 @@
     <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="2"/>
       <c r="B425" s="21" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C425" s="21"/>
       <c r="D425" s="21"/>
@@ -7822,7 +7819,7 @@
     <row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A426" s="2"/>
       <c r="B426" s="21" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C426" s="21"/>
       <c r="D426" s="21"/>
@@ -7831,7 +7828,7 @@
     <row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A427" s="2"/>
       <c r="B427" s="21" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C427" s="21"/>
       <c r="D427" s="21"/>
@@ -7840,7 +7837,7 @@
     <row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A428" s="2"/>
       <c r="B428" s="21" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="C428" s="21"/>
       <c r="D428" s="21"/>
@@ -7849,7 +7846,7 @@
     <row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A429" s="2"/>
       <c r="B429" s="21" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="C429" s="21"/>
       <c r="D429" s="21"/>
@@ -7858,28 +7855,28 @@
     <row r="430" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A430" s="2"/>
       <c r="B430" s="21" t="s">
+        <v>545</v>
+      </c>
+      <c r="C430" s="21" t="s">
         <v>546</v>
       </c>
-      <c r="C430" s="21" t="s">
+      <c r="D430" s="21" t="s">
         <v>547</v>
       </c>
-      <c r="D430" s="21" t="s">
+      <c r="E430" s="11" t="s">
         <v>548</v>
       </c>
-      <c r="E430" s="11" t="s">
+      <c r="F430" s="18" t="s">
         <v>549</v>
       </c>
-      <c r="F430" s="18" t="s">
+      <c r="G430" s="18" t="s">
         <v>550</v>
-      </c>
-      <c r="G430" s="18" t="s">
-        <v>551</v>
       </c>
     </row>
     <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="2"/>
       <c r="B431" s="21" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="C431" s="21"/>
       <c r="D431" s="21"/>
@@ -7888,7 +7885,7 @@
     <row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A432" s="2"/>
       <c r="B432" s="21" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="C432" s="21"/>
       <c r="D432" s="21"/>
@@ -7897,7 +7894,7 @@
     <row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A433" s="2"/>
       <c r="B433" s="21" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="C433" s="21"/>
       <c r="D433" s="21"/>
@@ -7906,7 +7903,7 @@
     <row r="434" customFormat="false" ht="36.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A434" s="2"/>
       <c r="B434" s="21" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C434" s="21"/>
       <c r="D434" s="21"/>
@@ -7915,13 +7912,13 @@
     <row r="435" customFormat="false" ht="67.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A435" s="2"/>
       <c r="B435" s="21" t="s">
+        <v>555</v>
+      </c>
+      <c r="C435" s="21" t="s">
         <v>556</v>
       </c>
-      <c r="C435" s="21" t="s">
+      <c r="D435" s="21" t="s">
         <v>557</v>
-      </c>
-      <c r="D435" s="21" t="s">
-        <v>558</v>
       </c>
       <c r="E435" s="11" t="s">
         <v>176</v>
@@ -7931,7 +7928,7 @@
     <row r="436" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A436" s="2"/>
       <c r="B436" s="21" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C436" s="21"/>
       <c r="D436" s="21"/>
@@ -7940,7 +7937,7 @@
     <row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A437" s="2"/>
       <c r="B437" s="21" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C437" s="21"/>
       <c r="D437" s="21"/>
@@ -7949,7 +7946,7 @@
     <row r="438" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A438" s="2"/>
       <c r="B438" s="21" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C438" s="21" t="s">
         <v>224</v>
@@ -7962,22 +7959,22 @@
     <row r="439" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A439" s="2"/>
       <c r="B439" s="21" t="s">
+        <v>561</v>
+      </c>
+      <c r="C439" s="21" t="s">
+        <v>519</v>
+      </c>
+      <c r="D439" s="21" t="s">
         <v>562</v>
       </c>
-      <c r="C439" s="21" t="s">
-        <v>520</v>
-      </c>
-      <c r="D439" s="21" t="s">
-        <v>563</v>
-      </c>
       <c r="E439" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A440" s="2"/>
       <c r="B440" s="21" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C440" s="21"/>
       <c r="D440" s="21"/>
@@ -7986,7 +7983,7 @@
     <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A441" s="2"/>
       <c r="B441" s="21" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="C441" s="21"/>
       <c r="D441" s="21"/>
@@ -7995,22 +7992,22 @@
     <row r="442" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A442" s="2"/>
       <c r="B442" s="21" t="s">
+        <v>565</v>
+      </c>
+      <c r="C442" s="21" t="s">
         <v>566</v>
       </c>
-      <c r="C442" s="21" t="s">
+      <c r="D442" s="21" t="s">
         <v>567</v>
       </c>
-      <c r="D442" s="21" t="s">
-        <v>568</v>
-      </c>
       <c r="E442" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A443" s="2"/>
       <c r="B443" s="21" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C443" s="21"/>
       <c r="D443" s="21"/>
@@ -8019,7 +8016,7 @@
     <row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A444" s="2"/>
       <c r="B444" s="21" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C444" s="21"/>
       <c r="D444" s="21"/>
@@ -8028,22 +8025,22 @@
     <row r="445" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="2"/>
       <c r="B445" s="21" t="s">
+        <v>570</v>
+      </c>
+      <c r="C445" s="21" t="s">
+        <v>536</v>
+      </c>
+      <c r="D445" s="21" t="s">
         <v>571</v>
       </c>
-      <c r="C445" s="21" t="s">
-        <v>537</v>
-      </c>
-      <c r="D445" s="21" t="s">
-        <v>572</v>
-      </c>
       <c r="E445" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="2"/>
       <c r="B446" s="21" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C446" s="21"/>
       <c r="D446" s="21"/>
@@ -8058,10 +8055,10 @@
     </row>
     <row r="448" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A448" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="B448" s="21" t="s">
         <v>574</v>
-      </c>
-      <c r="B448" s="21" t="s">
-        <v>575</v>
       </c>
       <c r="C448" s="21"/>
       <c r="D448" s="21"/>
@@ -8070,22 +8067,22 @@
     <row r="449" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="2"/>
       <c r="B449" s="21" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="C449" s="21" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="D449" s="21" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="E449" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A450" s="2"/>
       <c r="B450" s="21" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C450" s="21"/>
       <c r="D450" s="21"/>
@@ -8101,7 +8098,7 @@
     <row r="452" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A452" s="6"/>
       <c r="B452" s="22" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C452" s="23"/>
       <c r="D452" s="23"/>
@@ -8118,7 +8115,7 @@
     <row r="454" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A454" s="2"/>
       <c r="B454" s="21" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C454" s="21"/>
       <c r="D454" s="21"/>
@@ -8127,7 +8124,7 @@
     <row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A455" s="2"/>
       <c r="B455" s="21" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="C455" s="21"/>
       <c r="D455" s="21"/>
@@ -8136,7 +8133,7 @@
     <row r="456" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A456" s="2"/>
       <c r="B456" s="21" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C456" s="21"/>
       <c r="D456" s="21"/>
@@ -8145,7 +8142,7 @@
     <row r="457" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A457" s="2"/>
       <c r="B457" s="21" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C457" s="21"/>
       <c r="D457" s="21"/>
@@ -8154,16 +8151,16 @@
     <row r="458" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A458" s="2"/>
       <c r="B458" s="21" t="s">
+        <v>581</v>
+      </c>
+      <c r="C458" s="21" t="s">
+        <v>536</v>
+      </c>
+      <c r="D458" s="21" t="s">
         <v>582</v>
       </c>
-      <c r="C458" s="21" t="s">
-        <v>537</v>
-      </c>
-      <c r="D458" s="21" t="s">
-        <v>583</v>
-      </c>
       <c r="E458" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8176,7 +8173,7 @@
     <row r="460" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A460" s="6"/>
       <c r="B460" s="22" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="C460" s="23"/>
       <c r="D460" s="23"/>
@@ -8193,7 +8190,7 @@
     <row r="462" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A462" s="2"/>
       <c r="B462" s="21" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C462" s="21"/>
       <c r="D462" s="21"/>
@@ -8202,7 +8199,7 @@
     <row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A463" s="2"/>
       <c r="B463" s="21" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C463" s="21"/>
       <c r="D463" s="21"/>
@@ -8211,10 +8208,10 @@
     <row r="464" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A464" s="2"/>
       <c r="B464" s="21" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C464" s="21" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D464" s="21"/>
       <c r="E464" s="11"/>
@@ -8222,10 +8219,10 @@
     <row r="465" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="2"/>
       <c r="B465" s="21" t="s">
+        <v>587</v>
+      </c>
+      <c r="C465" s="21" t="s">
         <v>588</v>
-      </c>
-      <c r="C465" s="21" t="s">
-        <v>589</v>
       </c>
       <c r="D465" s="21"/>
       <c r="E465" s="11"/>
@@ -8233,10 +8230,10 @@
     <row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A466" s="2"/>
       <c r="B466" s="21" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C466" s="21" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="D466" s="21"/>
       <c r="E466" s="11"/>
@@ -8244,13 +8241,13 @@
     <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A467" s="2"/>
       <c r="B467" s="21" t="s">
+        <v>590</v>
+      </c>
+      <c r="C467" s="21" t="s">
         <v>591</v>
       </c>
-      <c r="C467" s="21" t="s">
+      <c r="D467" s="21" t="s">
         <v>592</v>
-      </c>
-      <c r="D467" s="21" t="s">
-        <v>593</v>
       </c>
       <c r="E467" s="11" t="s">
         <v>24</v>
@@ -8259,22 +8256,22 @@
     <row r="468" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A468" s="2"/>
       <c r="B468" s="21" t="s">
+        <v>593</v>
+      </c>
+      <c r="C468" s="21" t="s">
         <v>594</v>
       </c>
-      <c r="C468" s="21" t="s">
+      <c r="D468" s="21" t="s">
         <v>595</v>
       </c>
-      <c r="D468" s="21" t="s">
-        <v>596</v>
-      </c>
       <c r="E468" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="469" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A469" s="2"/>
       <c r="B469" s="21" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="C469" s="21"/>
       <c r="D469" s="21"/>
@@ -8290,17 +8287,17 @@
     <row r="471" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A471" s="6"/>
       <c r="B471" s="22" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="C471" s="23"/>
       <c r="D471" s="23" t="s">
+        <v>598</v>
+      </c>
+      <c r="E471" s="23" t="s">
+        <v>490</v>
+      </c>
+      <c r="F471" s="18" t="s">
         <v>599</v>
-      </c>
-      <c r="E471" s="23" t="s">
-        <v>491</v>
-      </c>
-      <c r="F471" s="18" t="s">
-        <v>600</v>
       </c>
     </row>
     <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8315,7 +8312,7 @@
     <row r="473" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A473" s="2"/>
       <c r="B473" s="21" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C473" s="21"/>
       <c r="D473" s="21"/>
@@ -8324,25 +8321,25 @@
     <row r="474" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A474" s="2"/>
       <c r="B474" s="21" t="s">
+        <v>601</v>
+      </c>
+      <c r="C474" s="21" t="s">
+        <v>509</v>
+      </c>
+      <c r="D474" s="21" t="s">
         <v>602</v>
       </c>
-      <c r="C474" s="21" t="s">
-        <v>510</v>
-      </c>
-      <c r="D474" s="21" t="s">
+      <c r="E474" s="11" t="s">
         <v>603</v>
       </c>
-      <c r="E474" s="11" t="s">
+      <c r="F474" s="18" t="s">
         <v>604</v>
-      </c>
-      <c r="F474" s="18" t="s">
-        <v>605</v>
       </c>
     </row>
     <row r="475" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A475" s="2"/>
       <c r="B475" s="21" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C475" s="21"/>
       <c r="D475" s="21"/>
@@ -8351,7 +8348,7 @@
     <row r="476" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A476" s="2"/>
       <c r="B476" s="21" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="C476" s="21"/>
       <c r="D476" s="21"/>
@@ -8360,7 +8357,7 @@
     <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A477" s="2"/>
       <c r="B477" s="21" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="C477" s="21"/>
       <c r="D477" s="21"/>
@@ -8369,10 +8366,10 @@
     <row r="478" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A478" s="2"/>
       <c r="B478" s="21" t="s">
+        <v>608</v>
+      </c>
+      <c r="C478" s="21" t="s">
         <v>609</v>
-      </c>
-      <c r="C478" s="21" t="s">
-        <v>610</v>
       </c>
       <c r="D478" s="21"/>
       <c r="E478" s="11"/>
@@ -8380,13 +8377,13 @@
     <row r="479" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A479" s="2"/>
       <c r="B479" s="21" t="s">
+        <v>610</v>
+      </c>
+      <c r="C479" s="21" t="s">
         <v>611</v>
       </c>
-      <c r="C479" s="21" t="s">
+      <c r="D479" s="21" t="s">
         <v>612</v>
-      </c>
-      <c r="D479" s="21" t="s">
-        <v>613</v>
       </c>
       <c r="E479" s="11" t="s">
         <v>176</v>
@@ -8401,10 +8398,10 @@
     </row>
     <row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A481" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="B481" s="21" t="s">
         <v>614</v>
-      </c>
-      <c r="B481" s="21" t="s">
-        <v>615</v>
       </c>
       <c r="C481" s="21"/>
       <c r="D481" s="21"/>
@@ -8413,7 +8410,7 @@
     <row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A482" s="2"/>
       <c r="B482" s="21" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="C482" s="21"/>
       <c r="D482" s="21"/>
@@ -8429,7 +8426,7 @@
     <row r="484" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A484" s="2"/>
       <c r="B484" s="21" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="C484" s="21"/>
       <c r="D484" s="21"/>
@@ -8438,7 +8435,7 @@
     <row r="485" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A485" s="2"/>
       <c r="B485" s="21" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="C485" s="21"/>
       <c r="D485" s="21"/>
@@ -8454,14 +8451,14 @@
     <row r="487" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A487" s="6"/>
       <c r="B487" s="22" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C487" s="23"/>
       <c r="D487" s="23" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="E487" s="8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8476,7 +8473,7 @@
     <row r="489" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A489" s="2"/>
       <c r="B489" s="21" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="C489" s="21"/>
       <c r="D489" s="21"/>
@@ -8485,35 +8482,35 @@
     <row r="490" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A490" s="2"/>
       <c r="B490" s="21" t="s">
+        <v>621</v>
+      </c>
+      <c r="C490" s="21" t="s">
         <v>622</v>
       </c>
-      <c r="C490" s="21" t="s">
+      <c r="D490" s="21" t="s">
         <v>623</v>
       </c>
-      <c r="D490" s="21" t="s">
-        <v>624</v>
-      </c>
       <c r="E490" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="491" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A491" s="2"/>
       <c r="B491" s="21" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="C491" s="21"/>
       <c r="D491" s="21" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="E491" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="492" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A492" s="2"/>
       <c r="B492" s="21" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="C492" s="21"/>
       <c r="D492" s="21"/>
@@ -8522,7 +8519,7 @@
     <row r="493" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A493" s="2"/>
       <c r="B493" s="21" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="C493" s="21" t="s">
         <v>276</v>
@@ -8534,13 +8531,13 @@
         <v>176</v>
       </c>
       <c r="F493" s="18" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A494" s="2"/>
       <c r="B494" s="21" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C494" s="21"/>
       <c r="D494" s="21"/>
@@ -8549,7 +8546,7 @@
     <row r="495" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A495" s="2"/>
       <c r="B495" s="21" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C495" s="21"/>
       <c r="D495" s="21"/>
@@ -8558,7 +8555,7 @@
     <row r="496" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A496" s="2"/>
       <c r="B496" s="21" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C496" s="21"/>
       <c r="D496" s="21"/>
@@ -8567,7 +8564,7 @@
     <row r="497" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A497" s="2"/>
       <c r="B497" s="21" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C497" s="21"/>
       <c r="D497" s="21"/>
@@ -8576,7 +8573,7 @@
     <row r="498" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A498" s="2"/>
       <c r="B498" s="21" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="C498" s="21"/>
       <c r="D498" s="21"/>
@@ -8585,7 +8582,7 @@
     <row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A499" s="2"/>
       <c r="B499" s="21" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C499" s="21"/>
       <c r="D499" s="21"/>
@@ -8594,7 +8591,7 @@
     <row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A500" s="2"/>
       <c r="B500" s="21" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="C500" s="21"/>
       <c r="D500" s="21"/>
@@ -8603,31 +8600,31 @@
     <row r="501" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A501" s="2"/>
       <c r="B501" s="21" t="s">
+        <v>636</v>
+      </c>
+      <c r="C501" s="21" t="s">
         <v>637</v>
       </c>
-      <c r="C501" s="21" t="s">
+      <c r="D501" s="21" t="s">
         <v>638</v>
       </c>
-      <c r="D501" s="21" t="s">
-        <v>639</v>
-      </c>
       <c r="E501" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="502" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A502" s="2"/>
       <c r="B502" s="21" t="s">
+        <v>639</v>
+      </c>
+      <c r="C502" s="21" t="s">
         <v>640</v>
       </c>
-      <c r="C502" s="21" t="s">
+      <c r="D502" s="21" t="s">
         <v>641</v>
       </c>
-      <c r="D502" s="21" t="s">
+      <c r="E502" s="11" t="s">
         <v>642</v>
-      </c>
-      <c r="E502" s="11" t="s">
-        <v>643</v>
       </c>
     </row>
     <row r="503" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8642,7 +8639,7 @@
         <v>236</v>
       </c>
       <c r="B504" s="21" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="C504" s="21"/>
       <c r="D504" s="21"/>
@@ -8651,7 +8648,7 @@
     <row r="505" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A505" s="2"/>
       <c r="B505" s="21" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="C505" s="21"/>
       <c r="D505" s="21"/>
@@ -8660,7 +8657,7 @@
     <row r="506" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A506" s="2"/>
       <c r="B506" s="21" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="C506" s="21"/>
       <c r="D506" s="21"/>
@@ -8669,7 +8666,7 @@
     <row r="507" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A507" s="2"/>
       <c r="B507" s="21" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="C507" s="21"/>
       <c r="D507" s="21"/>
@@ -8678,22 +8675,22 @@
     <row r="508" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A508" s="2"/>
       <c r="B508" s="21" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="C508" s="21" t="s">
+        <v>640</v>
+      </c>
+      <c r="D508" s="21" t="s">
         <v>641</v>
       </c>
-      <c r="D508" s="21" t="s">
+      <c r="E508" s="11" t="s">
         <v>642</v>
-      </c>
-      <c r="E508" s="11" t="s">
-        <v>643</v>
       </c>
     </row>
     <row r="509" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A509" s="2"/>
       <c r="B509" s="21" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="C509" s="21"/>
       <c r="D509" s="21"/>
@@ -8702,7 +8699,7 @@
     <row r="510" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A510" s="2"/>
       <c r="B510" s="21" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="C510" s="21"/>
       <c r="D510" s="21"/>
@@ -8711,7 +8708,7 @@
     <row r="511" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A511" s="2"/>
       <c r="B511" s="21" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="C511" s="21"/>
       <c r="D511" s="21"/>
@@ -8720,7 +8717,7 @@
     <row r="512" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A512" s="2"/>
       <c r="B512" s="21" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="C512" s="21"/>
       <c r="D512" s="21"/>
@@ -8729,10 +8726,10 @@
     <row r="513" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A513" s="2"/>
       <c r="B513" s="21" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="C513" s="21" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D513" s="21"/>
       <c r="E513" s="11"/>
@@ -8740,7 +8737,7 @@
     <row r="514" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A514" s="2"/>
       <c r="B514" s="21" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="C514" s="21"/>
       <c r="D514" s="21"/>
@@ -8749,7 +8746,7 @@
     <row r="515" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A515" s="2"/>
       <c r="B515" s="21" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="C515" s="21"/>
       <c r="D515" s="21"/>
@@ -8758,7 +8755,7 @@
     <row r="516" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A516" s="2"/>
       <c r="B516" s="21" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="C516" s="21"/>
       <c r="D516" s="21"/>
@@ -8767,7 +8764,7 @@
     <row r="517" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A517" s="2"/>
       <c r="B517" s="21" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="C517" s="21"/>
       <c r="D517" s="21"/>
@@ -8776,7 +8773,7 @@
     <row r="518" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A518" s="2"/>
       <c r="B518" s="21" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="C518" s="21"/>
       <c r="D518" s="21"/>
@@ -8785,7 +8782,7 @@
     <row r="519" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A519" s="2"/>
       <c r="B519" s="21" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="C519" s="21"/>
       <c r="D519" s="21"/>
@@ -8794,28 +8791,28 @@
     <row r="520" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A520" s="2"/>
       <c r="B520" s="21" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C520" s="21" t="s">
         <v>276</v>
       </c>
       <c r="D520" s="21" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="E520" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="521" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A521" s="2"/>
       <c r="B521" s="21" t="s">
+        <v>661</v>
+      </c>
+      <c r="C521" s="21" t="s">
         <v>662</v>
       </c>
-      <c r="C521" s="21" t="s">
+      <c r="D521" s="21" t="s">
         <v>663</v>
-      </c>
-      <c r="D521" s="21" t="s">
-        <v>664</v>
       </c>
       <c r="E521" s="11" t="s">
         <v>176</v>
@@ -8824,7 +8821,7 @@
     <row r="522" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A522" s="2"/>
       <c r="B522" s="21" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="C522" s="21"/>
       <c r="D522" s="21"/>
@@ -8839,10 +8836,10 @@
     </row>
     <row r="524" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A524" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B524" s="21" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="C524" s="21"/>
       <c r="D524" s="21"/>
@@ -8851,7 +8848,7 @@
     <row r="525" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A525" s="2"/>
       <c r="B525" s="21" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="C525" s="21"/>
       <c r="D525" s="21"/>
@@ -8860,7 +8857,7 @@
     <row r="526" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A526" s="2"/>
       <c r="B526" s="21" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="C526" s="21"/>
       <c r="D526" s="21"/>
@@ -8869,16 +8866,16 @@
     <row r="527" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A527" s="2"/>
       <c r="B527" s="21" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C527" s="21" t="s">
+        <v>640</v>
+      </c>
+      <c r="D527" s="21" t="s">
         <v>641</v>
       </c>
-      <c r="D527" s="21" t="s">
+      <c r="E527" s="11" t="s">
         <v>642</v>
-      </c>
-      <c r="E527" s="11" t="s">
-        <v>643</v>
       </c>
     </row>
     <row r="528" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8891,7 +8888,7 @@
     <row r="529" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A529" s="2"/>
       <c r="B529" s="21" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="C529" s="21"/>
       <c r="D529" s="21"/>
@@ -8900,7 +8897,7 @@
     <row r="530" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A530" s="32"/>
       <c r="B530" s="33" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="C530" s="33"/>
       <c r="D530" s="33"/>

</xml_diff>